<commit_message>
Updates (not sure content)
</commit_message>
<xml_diff>
--- a/data/thesis_sediment master (raw).xlsx
+++ b/data/thesis_sediment master (raw).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mailsfsu-my.sharepoint.com/personal/924318106_sfsu_edu/Documents/ProjectData/GitHub/DepositionSFB/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1055" documentId="8_{625E32F6-7E88-4DA8-AE14-1AD01B36A6CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5149995F-2C5B-416B-AEC0-3906876A727C}"/>
+  <xr:revisionPtr revIDLastSave="1056" documentId="8_{625E32F6-7E88-4DA8-AE14-1AD01B36A6CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6C21FA63-8EF5-4CBC-95A0-2599EEED2BE9}"/>
   <bookViews>
-    <workbookView xWindow="-28935" yWindow="-4095" windowWidth="29070" windowHeight="16470" xr2:uid="{7E299392-FF5E-4B95-B4B7-FEDF7BC05BEF}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13152" xr2:uid="{7E299392-FF5E-4B95-B4B7-FEDF7BC05BEF}"/>
   </bookViews>
   <sheets>
     <sheet name="sediment master (raw)" sheetId="1" r:id="rId1"/>
@@ -142,7 +142,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10454" uniqueCount="364">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10455" uniqueCount="364">
   <si>
     <t>Data Check 1</t>
   </si>
@@ -2158,7 +2158,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E195799A-9D02-4A88-AC8B-3DBDF1F16FC3}">
-  <dimension ref="A1:S2162"/>
+  <dimension ref="A1:X2162"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.33203125" customWidth="1"/>
@@ -68407,7 +68407,7 @@
         <v>5.31</v>
       </c>
     </row>
-    <row r="1425" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="1425" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A1425" t="s">
         <v>289</v>
       </c>
@@ -68439,7 +68439,7 @@
         <v>5.31</v>
       </c>
     </row>
-    <row r="1426" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="1426" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A1426" t="s">
         <v>289</v>
       </c>
@@ -68471,7 +68471,7 @@
         <v>5.31</v>
       </c>
     </row>
-    <row r="1427" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="1427" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A1427" t="s">
         <v>329</v>
       </c>
@@ -68518,7 +68518,7 @@
         <v>9.7731999999999992</v>
       </c>
     </row>
-    <row r="1428" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="1428" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A1428" t="s">
         <v>329</v>
       </c>
@@ -68565,7 +68565,7 @@
         <v>9.6484699999999997</v>
       </c>
     </row>
-    <row r="1429" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="1429" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A1429" t="s">
         <v>329</v>
       </c>
@@ -68612,7 +68612,7 @@
         <v>9.9962099999999996</v>
       </c>
     </row>
-    <row r="1430" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="1430" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A1430" t="s">
         <v>329</v>
       </c>
@@ -68659,7 +68659,7 @@
         <v>9.68384</v>
       </c>
     </row>
-    <row r="1431" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="1431" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A1431" t="s">
         <v>329</v>
       </c>
@@ -68706,7 +68706,7 @@
         <v>9.6142400000000006</v>
       </c>
     </row>
-    <row r="1432" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="1432" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A1432" t="s">
         <v>329</v>
       </c>
@@ -68753,7 +68753,7 @@
         <v>9.5764999999999993</v>
       </c>
     </row>
-    <row r="1433" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="1433" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A1433" t="s">
         <v>329</v>
       </c>
@@ -68800,7 +68800,7 @@
         <v>5.7963699999999996</v>
       </c>
     </row>
-    <row r="1434" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="1434" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A1434" t="s">
         <v>329</v>
       </c>
@@ -68847,7 +68847,7 @@
         <v>5.7477299999999998</v>
       </c>
     </row>
-    <row r="1435" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="1435" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A1435" t="s">
         <v>329</v>
       </c>
@@ -68893,8 +68893,11 @@
       <c r="P1435">
         <v>5.7550699999999999</v>
       </c>
-    </row>
-    <row r="1436" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="X1435" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="1436" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A1436" t="s">
         <v>329</v>
       </c>
@@ -68941,7 +68944,7 @@
         <v>5.7636599999999998</v>
       </c>
     </row>
-    <row r="1437" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="1437" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A1437" t="s">
         <v>329</v>
       </c>
@@ -68988,7 +68991,7 @@
         <v>5.7142400000000002</v>
       </c>
     </row>
-    <row r="1438" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="1438" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A1438" t="s">
         <v>329</v>
       </c>
@@ -69035,7 +69038,7 @@
         <v>5.7049300000000001</v>
       </c>
     </row>
-    <row r="1439" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="1439" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A1439" t="s">
         <v>329</v>
       </c>
@@ -69082,7 +69085,7 @@
         <v>5.7422399999999998</v>
       </c>
     </row>
-    <row r="1440" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="1440" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A1440" t="s">
         <v>329</v>
       </c>

</xml_diff>

<commit_message>
Mistake-don't pay attention to it-have to correct with field notes tomorrow
</commit_message>
<xml_diff>
--- a/data/thesis_sediment master (raw).xlsx
+++ b/data/thesis_sediment master (raw).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mailsfsu-my.sharepoint.com/personal/924318106_sfsu_edu/Documents/ProjectData/GitHub/DepositionSFB/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1056" documentId="8_{625E32F6-7E88-4DA8-AE14-1AD01B36A6CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6C21FA63-8EF5-4CBC-95A0-2599EEED2BE9}"/>
+  <xr:revisionPtr revIDLastSave="1064" documentId="8_{625E32F6-7E88-4DA8-AE14-1AD01B36A6CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DEB57D68-48E8-4E83-A8E1-A5EA9C53D82B}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13152" xr2:uid="{7E299392-FF5E-4B95-B4B7-FEDF7BC05BEF}"/>
   </bookViews>
@@ -1759,7 +1759,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -1779,7 +1779,6 @@
     <xf numFmtId="14" fontId="0" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="166" fontId="0" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
@@ -1839,6 +1838,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -59168,7 +59171,7 @@
       <c r="G1224" t="s">
         <v>24</v>
       </c>
-      <c r="H1224" s="13">
+      <c r="H1224">
         <v>0.44655</v>
       </c>
       <c r="I1224" s="1">
@@ -71297,7 +71300,7 @@
       <c r="I1488" s="1">
         <v>46100</v>
       </c>
-      <c r="J1488" s="14">
+      <c r="J1488" s="13">
         <v>5.0726000000000004</v>
       </c>
       <c r="K1488" s="1">
@@ -71829,7 +71832,7 @@
       <c r="O1499" t="s">
         <v>359</v>
       </c>
-      <c r="P1499" s="15">
+      <c r="P1499" s="14">
         <v>55.100999999999999</v>
       </c>
     </row>
@@ -74260,7 +74263,7 @@
       <c r="O1552" t="s">
         <v>360</v>
       </c>
-      <c r="P1552" s="13">
+      <c r="P1552">
         <v>5.8418700000000001</v>
       </c>
     </row>
@@ -74307,7 +74310,7 @@
       <c r="O1553" t="s">
         <v>360</v>
       </c>
-      <c r="P1553" s="14">
+      <c r="P1553" s="13">
         <v>5.9027000000000003</v>
       </c>
     </row>
@@ -76599,7 +76602,7 @@
       <c r="I1601" s="1">
         <v>46087</v>
       </c>
-      <c r="J1601" s="16">
+      <c r="J1601" s="15">
         <v>5.0903</v>
       </c>
       <c r="K1601" s="1">
@@ -76799,7 +76802,7 @@
       <c r="I1605" s="1">
         <v>46087</v>
       </c>
-      <c r="J1605" s="16">
+      <c r="J1605" s="15">
         <v>5.1108599999999997</v>
       </c>
       <c r="K1605" s="1">
@@ -76814,7 +76817,7 @@
       <c r="O1605" t="s">
         <v>361</v>
       </c>
-      <c r="P1605" s="14">
+      <c r="P1605" s="13">
         <v>5.6449999999999996</v>
       </c>
       <c r="S1605" t="s">
@@ -79768,7 +79771,7 @@
       <c r="I1678" s="1">
         <v>46129</v>
       </c>
-      <c r="J1678" s="15">
+      <c r="J1678" s="14">
         <v>2.0329999999999999</v>
       </c>
       <c r="K1678" s="1">
@@ -80000,7 +80003,7 @@
       <c r="M1683">
         <v>5.31</v>
       </c>
-      <c r="P1683" s="15">
+      <c r="P1683" s="14">
         <v>37.203000000000003</v>
       </c>
       <c r="S1683" t="s">

</xml_diff>

<commit_message>
Transferred data into calc sheet
NEED to do a triple check of the data for individual variations, such as proportions of filter sizes, rubber band surface area etc. Will require a lab visit when measuring LOI and sorting the samples
</commit_message>
<xml_diff>
--- a/data/thesis_sediment master (raw).xlsx
+++ b/data/thesis_sediment master (raw).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mailsfsu-my.sharepoint.com/personal/924318106_sfsu_edu/Documents/ProjectData/GitHub/DepositionSFB/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1376" documentId="8_{625E32F6-7E88-4DA8-AE14-1AD01B36A6CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2898962B-5868-403B-8A56-22707E37ECD7}"/>
+  <xr:revisionPtr revIDLastSave="1443" documentId="8_{625E32F6-7E88-4DA8-AE14-1AD01B36A6CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{14024D4C-7538-430D-BA2D-C161C67B0338}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-4080" windowWidth="29040" windowHeight="16440" xr2:uid="{7E299392-FF5E-4B95-B4B7-FEDF7BC05BEF}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{7E299392-FF5E-4B95-B4B7-FEDF7BC05BEF}"/>
   </bookViews>
   <sheets>
     <sheet name="sediment master (raw)" sheetId="1" r:id="rId1"/>
@@ -1993,7 +1993,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -2018,7 +2018,6 @@
     <xf numFmtId="166" fontId="0" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -11741,47 +11740,47 @@
         <v>27</v>
       </c>
     </row>
-    <row r="201" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A201" s="1">
+    <row r="201" spans="1:19" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A201" s="10">
         <v>46092</v>
       </c>
-      <c r="C201" t="s">
+      <c r="C201" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="D201" t="s">
+      <c r="D201" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="E201">
-        <v>2</v>
-      </c>
-      <c r="G201" t="s">
+      <c r="E201" s="9">
+        <v>2</v>
+      </c>
+      <c r="G201" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="H201">
+      <c r="H201" s="9">
         <v>0.43260999999999999</v>
       </c>
-      <c r="I201" s="1" t="s">
+      <c r="I201" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="J201">
+      <c r="J201" s="9">
         <v>6.6252800000000001</v>
       </c>
-      <c r="K201" s="1" t="s">
+      <c r="K201" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="L201">
-        <v>63.617251160000002</v>
-      </c>
-      <c r="M201">
-        <v>5.31</v>
-      </c>
-      <c r="N201">
-        <v>1</v>
-      </c>
-      <c r="P201">
+      <c r="L201" s="9">
+        <v>63.617251160000002</v>
+      </c>
+      <c r="M201" s="9">
+        <v>5.31</v>
+      </c>
+      <c r="N201" s="9">
+        <v>1</v>
+      </c>
+      <c r="P201" s="9">
         <v>8.5910899999999994</v>
       </c>
-      <c r="S201" t="s">
+      <c r="S201" s="9" t="s">
         <v>63</v>
       </c>
     </row>
@@ -62659,6 +62658,9 @@
       <c r="M1289">
         <v>5.31</v>
       </c>
+      <c r="N1289">
+        <v>1</v>
+      </c>
       <c r="O1289" t="s">
         <v>423</v>
       </c>
@@ -62709,6 +62711,9 @@
       <c r="M1290">
         <v>5.31</v>
       </c>
+      <c r="N1290">
+        <v>1</v>
+      </c>
       <c r="O1290" t="s">
         <v>423</v>
       </c>
@@ -62759,6 +62764,9 @@
       <c r="M1291">
         <v>5.31</v>
       </c>
+      <c r="N1291">
+        <v>1</v>
+      </c>
       <c r="O1291" t="s">
         <v>423</v>
       </c>
@@ -62809,6 +62817,9 @@
       <c r="M1292">
         <v>5.31</v>
       </c>
+      <c r="N1292">
+        <v>1</v>
+      </c>
       <c r="O1292" t="s">
         <v>423</v>
       </c>
@@ -62859,6 +62870,9 @@
       <c r="M1293">
         <v>5.31</v>
       </c>
+      <c r="N1293">
+        <v>1</v>
+      </c>
       <c r="O1293" t="s">
         <v>423</v>
       </c>
@@ -62909,6 +62923,9 @@
       <c r="M1294">
         <v>5.31</v>
       </c>
+      <c r="N1294">
+        <v>1</v>
+      </c>
       <c r="O1294" t="s">
         <v>423</v>
       </c>
@@ -62959,6 +62976,9 @@
       <c r="M1295">
         <v>5.31</v>
       </c>
+      <c r="N1295">
+        <v>1</v>
+      </c>
       <c r="O1295" t="s">
         <v>423</v>
       </c>
@@ -63009,6 +63029,9 @@
       <c r="M1296">
         <v>5.31</v>
       </c>
+      <c r="N1296">
+        <v>1</v>
+      </c>
       <c r="O1296" t="s">
         <v>423</v>
       </c>
@@ -63059,6 +63082,9 @@
       <c r="M1297">
         <v>5.31</v>
       </c>
+      <c r="N1297">
+        <v>1</v>
+      </c>
       <c r="O1297" t="s">
         <v>423</v>
       </c>
@@ -63109,6 +63135,9 @@
       <c r="M1298">
         <v>5.31</v>
       </c>
+      <c r="N1298">
+        <v>1</v>
+      </c>
       <c r="O1298" t="s">
         <v>423</v>
       </c>
@@ -63159,6 +63188,9 @@
       <c r="M1299">
         <v>5.31</v>
       </c>
+      <c r="N1299">
+        <v>1</v>
+      </c>
       <c r="O1299" t="s">
         <v>423</v>
       </c>
@@ -63209,6 +63241,9 @@
       <c r="M1300">
         <v>5.31</v>
       </c>
+      <c r="N1300">
+        <v>1</v>
+      </c>
       <c r="O1300" t="s">
         <v>423</v>
       </c>
@@ -63259,6 +63294,9 @@
       <c r="M1301">
         <v>5.31</v>
       </c>
+      <c r="N1301">
+        <v>1</v>
+      </c>
       <c r="O1301" t="s">
         <v>423</v>
       </c>
@@ -63309,6 +63347,9 @@
       <c r="M1302">
         <v>5.31</v>
       </c>
+      <c r="N1302">
+        <v>1</v>
+      </c>
       <c r="O1302" t="s">
         <v>423</v>
       </c>
@@ -63359,6 +63400,9 @@
       <c r="M1303">
         <v>5.31</v>
       </c>
+      <c r="N1303">
+        <v>1</v>
+      </c>
       <c r="O1303" t="s">
         <v>423</v>
       </c>
@@ -63409,6 +63453,9 @@
       <c r="M1304">
         <v>5.31</v>
       </c>
+      <c r="N1304">
+        <v>1</v>
+      </c>
       <c r="O1304" t="s">
         <v>423</v>
       </c>
@@ -63459,6 +63506,9 @@
       <c r="M1305">
         <v>5.31</v>
       </c>
+      <c r="N1305">
+        <v>1</v>
+      </c>
       <c r="O1305" t="s">
         <v>423</v>
       </c>
@@ -63509,6 +63559,9 @@
       <c r="M1306">
         <v>5.31</v>
       </c>
+      <c r="N1306">
+        <v>1</v>
+      </c>
       <c r="O1306" t="s">
         <v>423</v>
       </c>
@@ -63559,6 +63612,9 @@
       <c r="M1307">
         <v>5.31</v>
       </c>
+      <c r="N1307">
+        <v>1</v>
+      </c>
       <c r="O1307" t="s">
         <v>423</v>
       </c>
@@ -63609,6 +63665,9 @@
       <c r="M1308">
         <v>5.31</v>
       </c>
+      <c r="N1308">
+        <v>1</v>
+      </c>
       <c r="O1308" t="s">
         <v>423</v>
       </c>
@@ -63659,6 +63718,9 @@
       <c r="M1309">
         <v>5.31</v>
       </c>
+      <c r="N1309">
+        <v>1</v>
+      </c>
       <c r="O1309" t="s">
         <v>423</v>
       </c>
@@ -63709,6 +63771,9 @@
       <c r="M1310">
         <v>5.31</v>
       </c>
+      <c r="N1310">
+        <v>1</v>
+      </c>
       <c r="O1310" t="s">
         <v>423</v>
       </c>
@@ -63759,6 +63824,9 @@
       <c r="M1311">
         <v>5.31</v>
       </c>
+      <c r="N1311">
+        <v>1</v>
+      </c>
       <c r="O1311" t="s">
         <v>423</v>
       </c>
@@ -63809,6 +63877,9 @@
       <c r="M1312">
         <v>5.31</v>
       </c>
+      <c r="N1312">
+        <v>1</v>
+      </c>
       <c r="O1312" t="s">
         <v>423</v>
       </c>
@@ -63859,6 +63930,9 @@
       <c r="M1313">
         <v>5.31</v>
       </c>
+      <c r="N1313">
+        <v>1</v>
+      </c>
       <c r="O1313" t="s">
         <v>423</v>
       </c>
@@ -63909,6 +63983,9 @@
       <c r="M1314">
         <v>5.31</v>
       </c>
+      <c r="N1314">
+        <v>1</v>
+      </c>
       <c r="O1314" t="s">
         <v>423</v>
       </c>
@@ -63959,6 +64036,9 @@
       <c r="M1315">
         <v>5.31</v>
       </c>
+      <c r="N1315">
+        <v>1</v>
+      </c>
       <c r="O1315" t="s">
         <v>423</v>
       </c>
@@ -64009,6 +64089,9 @@
       <c r="M1316">
         <v>5.31</v>
       </c>
+      <c r="N1316">
+        <v>1</v>
+      </c>
       <c r="O1316" t="s">
         <v>423</v>
       </c>
@@ -64059,6 +64142,9 @@
       <c r="M1317">
         <v>5.31</v>
       </c>
+      <c r="N1317">
+        <v>1</v>
+      </c>
       <c r="O1317" t="s">
         <v>423</v>
       </c>
@@ -64109,6 +64195,9 @@
       <c r="M1318">
         <v>5.31</v>
       </c>
+      <c r="N1318">
+        <v>1</v>
+      </c>
       <c r="O1318" t="s">
         <v>423</v>
       </c>
@@ -64159,6 +64248,9 @@
       <c r="M1319">
         <v>5.31</v>
       </c>
+      <c r="N1319">
+        <v>1</v>
+      </c>
       <c r="O1319" t="s">
         <v>423</v>
       </c>
@@ -64209,6 +64301,9 @@
       <c r="M1320">
         <v>5.31</v>
       </c>
+      <c r="N1320">
+        <v>1</v>
+      </c>
       <c r="O1320" t="s">
         <v>423</v>
       </c>
@@ -64259,6 +64354,9 @@
       <c r="M1321">
         <v>5.31</v>
       </c>
+      <c r="N1321">
+        <v>1</v>
+      </c>
       <c r="O1321" t="s">
         <v>423</v>
       </c>
@@ -64309,6 +64407,9 @@
       <c r="M1322">
         <v>5.31</v>
       </c>
+      <c r="N1322">
+        <v>1</v>
+      </c>
       <c r="O1322" t="s">
         <v>423</v>
       </c>
@@ -64359,6 +64460,9 @@
       <c r="M1323">
         <v>5.31</v>
       </c>
+      <c r="N1323">
+        <v>1</v>
+      </c>
       <c r="O1323" t="s">
         <v>423</v>
       </c>
@@ -64409,6 +64513,9 @@
       <c r="M1324">
         <v>5.31</v>
       </c>
+      <c r="N1324">
+        <v>1</v>
+      </c>
       <c r="O1324" t="s">
         <v>423</v>
       </c>
@@ -64459,6 +64566,9 @@
       <c r="M1325">
         <v>5.31</v>
       </c>
+      <c r="N1325">
+        <v>1</v>
+      </c>
       <c r="O1325" t="s">
         <v>423</v>
       </c>
@@ -64509,6 +64619,9 @@
       <c r="M1326">
         <v>5.31</v>
       </c>
+      <c r="N1326">
+        <v>1</v>
+      </c>
       <c r="O1326" t="s">
         <v>423</v>
       </c>
@@ -64559,6 +64672,9 @@
       <c r="M1327">
         <v>5.31</v>
       </c>
+      <c r="N1327">
+        <v>1</v>
+      </c>
       <c r="O1327" t="s">
         <v>423</v>
       </c>
@@ -64609,6 +64725,9 @@
       <c r="M1328">
         <v>5.31</v>
       </c>
+      <c r="N1328">
+        <v>1</v>
+      </c>
       <c r="O1328" t="s">
         <v>423</v>
       </c>
@@ -64659,6 +64778,9 @@
       <c r="M1329">
         <v>5.31</v>
       </c>
+      <c r="N1329">
+        <v>1</v>
+      </c>
       <c r="O1329" t="s">
         <v>423</v>
       </c>
@@ -64709,6 +64831,9 @@
       <c r="M1330">
         <v>5.31</v>
       </c>
+      <c r="N1330">
+        <v>1</v>
+      </c>
       <c r="O1330" t="s">
         <v>423</v>
       </c>
@@ -64923,6 +65048,9 @@
       <c r="M1335">
         <v>5.31</v>
       </c>
+      <c r="N1335">
+        <v>1</v>
+      </c>
       <c r="O1335" t="s">
         <v>424</v>
       </c>
@@ -64973,6 +65101,9 @@
       <c r="M1336">
         <v>5.31</v>
       </c>
+      <c r="N1336">
+        <v>1</v>
+      </c>
       <c r="O1336" t="s">
         <v>424</v>
       </c>
@@ -65023,6 +65154,9 @@
       <c r="M1337">
         <v>5.31</v>
       </c>
+      <c r="N1337">
+        <v>1</v>
+      </c>
       <c r="O1337" t="s">
         <v>424</v>
       </c>
@@ -65073,6 +65207,9 @@
       <c r="M1338">
         <v>5.31</v>
       </c>
+      <c r="N1338">
+        <v>1</v>
+      </c>
       <c r="O1338" t="s">
         <v>424</v>
       </c>
@@ -65123,6 +65260,9 @@
       <c r="M1339">
         <v>5.31</v>
       </c>
+      <c r="N1339">
+        <v>1</v>
+      </c>
       <c r="O1339" t="s">
         <v>424</v>
       </c>
@@ -65173,6 +65313,9 @@
       <c r="M1340">
         <v>5.31</v>
       </c>
+      <c r="N1340">
+        <v>1</v>
+      </c>
       <c r="O1340" t="s">
         <v>424</v>
       </c>
@@ -65223,6 +65366,9 @@
       <c r="M1341">
         <v>5.31</v>
       </c>
+      <c r="N1341">
+        <v>1</v>
+      </c>
       <c r="O1341" t="s">
         <v>424</v>
       </c>
@@ -65273,6 +65419,9 @@
       <c r="M1342">
         <v>5.31</v>
       </c>
+      <c r="N1342">
+        <v>1</v>
+      </c>
       <c r="O1342" t="s">
         <v>424</v>
       </c>
@@ -65323,6 +65472,9 @@
       <c r="M1343">
         <v>5.31</v>
       </c>
+      <c r="N1343">
+        <v>1</v>
+      </c>
       <c r="O1343" t="s">
         <v>424</v>
       </c>
@@ -65373,6 +65525,9 @@
       <c r="M1344" s="9">
         <v>5.31</v>
       </c>
+      <c r="N1344">
+        <v>1</v>
+      </c>
       <c r="O1344" t="s">
         <v>424</v>
       </c>
@@ -65423,6 +65578,9 @@
       <c r="M1345" s="9">
         <v>5.31</v>
       </c>
+      <c r="N1345">
+        <v>1</v>
+      </c>
       <c r="O1345" t="s">
         <v>424</v>
       </c>
@@ -65473,6 +65631,9 @@
       <c r="M1346" s="9">
         <v>5.31</v>
       </c>
+      <c r="N1346">
+        <v>1</v>
+      </c>
       <c r="O1346" t="s">
         <v>424</v>
       </c>
@@ -65523,6 +65684,9 @@
       <c r="M1347">
         <v>5.31</v>
       </c>
+      <c r="N1347">
+        <v>1</v>
+      </c>
       <c r="O1347" t="s">
         <v>424</v>
       </c>
@@ -65573,6 +65737,9 @@
       <c r="M1348">
         <v>5.31</v>
       </c>
+      <c r="N1348">
+        <v>1</v>
+      </c>
       <c r="O1348" t="s">
         <v>424</v>
       </c>
@@ -65623,6 +65790,9 @@
       <c r="M1349" s="9">
         <v>5.31</v>
       </c>
+      <c r="N1349">
+        <v>1</v>
+      </c>
       <c r="O1349" t="s">
         <v>424</v>
       </c>
@@ -65673,6 +65843,9 @@
       <c r="M1350">
         <v>5.31</v>
       </c>
+      <c r="N1350">
+        <v>1</v>
+      </c>
       <c r="O1350" t="s">
         <v>424</v>
       </c>
@@ -65723,6 +65896,9 @@
       <c r="M1351" s="9">
         <v>5.31</v>
       </c>
+      <c r="N1351">
+        <v>1</v>
+      </c>
       <c r="O1351" t="s">
         <v>424</v>
       </c>
@@ -65773,6 +65949,9 @@
       <c r="M1352">
         <v>5.31</v>
       </c>
+      <c r="N1352">
+        <v>1</v>
+      </c>
       <c r="O1352" t="s">
         <v>424</v>
       </c>
@@ -65823,6 +66002,9 @@
       <c r="M1353">
         <v>5.31</v>
       </c>
+      <c r="N1353">
+        <v>1</v>
+      </c>
       <c r="O1353" t="s">
         <v>424</v>
       </c>
@@ -65873,6 +66055,9 @@
       <c r="M1354">
         <v>5.31</v>
       </c>
+      <c r="N1354">
+        <v>1</v>
+      </c>
       <c r="O1354" t="s">
         <v>424</v>
       </c>
@@ -65923,6 +66108,9 @@
       <c r="M1355">
         <v>5.31</v>
       </c>
+      <c r="N1355">
+        <v>1</v>
+      </c>
       <c r="O1355" t="s">
         <v>424</v>
       </c>
@@ -65973,6 +66161,9 @@
       <c r="M1356">
         <v>5.31</v>
       </c>
+      <c r="N1356">
+        <v>1</v>
+      </c>
       <c r="O1356" t="s">
         <v>424</v>
       </c>
@@ -66023,6 +66214,9 @@
       <c r="M1357">
         <v>5.31</v>
       </c>
+      <c r="N1357">
+        <v>1</v>
+      </c>
       <c r="O1357" t="s">
         <v>424</v>
       </c>
@@ -66073,6 +66267,9 @@
       <c r="M1358">
         <v>5.31</v>
       </c>
+      <c r="N1358">
+        <v>1</v>
+      </c>
       <c r="O1358" t="s">
         <v>424</v>
       </c>
@@ -66123,6 +66320,9 @@
       <c r="M1359">
         <v>5.31</v>
       </c>
+      <c r="N1359">
+        <v>1</v>
+      </c>
       <c r="O1359" t="s">
         <v>424</v>
       </c>
@@ -66173,6 +66373,9 @@
       <c r="M1360">
         <v>5.31</v>
       </c>
+      <c r="N1360">
+        <v>1</v>
+      </c>
       <c r="O1360" t="s">
         <v>424</v>
       </c>
@@ -66223,6 +66426,9 @@
       <c r="M1361">
         <v>5.31</v>
       </c>
+      <c r="N1361">
+        <v>1</v>
+      </c>
       <c r="O1361" t="s">
         <v>424</v>
       </c>
@@ -66273,6 +66479,9 @@
       <c r="M1362">
         <v>5.31</v>
       </c>
+      <c r="N1362">
+        <v>1</v>
+      </c>
       <c r="O1362" t="s">
         <v>424</v>
       </c>
@@ -66323,6 +66532,9 @@
       <c r="M1363">
         <v>5.31</v>
       </c>
+      <c r="N1363">
+        <v>1</v>
+      </c>
       <c r="O1363" t="s">
         <v>424</v>
       </c>
@@ -66373,6 +66585,9 @@
       <c r="M1364">
         <v>5.31</v>
       </c>
+      <c r="N1364">
+        <v>1</v>
+      </c>
       <c r="O1364" t="s">
         <v>424</v>
       </c>
@@ -66423,6 +66638,9 @@
       <c r="M1365">
         <v>5.31</v>
       </c>
+      <c r="N1365">
+        <v>1</v>
+      </c>
       <c r="O1365" t="s">
         <v>424</v>
       </c>
@@ -66473,6 +66691,9 @@
       <c r="M1366">
         <v>5.31</v>
       </c>
+      <c r="N1366">
+        <v>1</v>
+      </c>
       <c r="O1366" t="s">
         <v>424</v>
       </c>
@@ -66523,6 +66744,9 @@
       <c r="M1367">
         <v>5.31</v>
       </c>
+      <c r="N1367">
+        <v>1</v>
+      </c>
       <c r="O1367" t="s">
         <v>424</v>
       </c>
@@ -66573,6 +66797,9 @@
       <c r="M1368">
         <v>5.31</v>
       </c>
+      <c r="N1368">
+        <v>1</v>
+      </c>
       <c r="O1368" t="s">
         <v>424</v>
       </c>
@@ -66623,6 +66850,9 @@
       <c r="M1369">
         <v>5.31</v>
       </c>
+      <c r="N1369">
+        <v>1</v>
+      </c>
       <c r="O1369" t="s">
         <v>424</v>
       </c>
@@ -66673,6 +66903,9 @@
       <c r="M1370">
         <v>5.31</v>
       </c>
+      <c r="N1370">
+        <v>1</v>
+      </c>
       <c r="O1370" t="s">
         <v>424</v>
       </c>
@@ -66723,6 +66956,9 @@
       <c r="M1371">
         <v>5.31</v>
       </c>
+      <c r="N1371">
+        <v>1</v>
+      </c>
       <c r="O1371" t="s">
         <v>424</v>
       </c>
@@ -66773,6 +67009,9 @@
       <c r="M1372">
         <v>5.31</v>
       </c>
+      <c r="N1372">
+        <v>1</v>
+      </c>
       <c r="O1372" t="s">
         <v>424</v>
       </c>
@@ -66823,6 +67062,9 @@
       <c r="M1373">
         <v>5.31</v>
       </c>
+      <c r="N1373">
+        <v>1</v>
+      </c>
       <c r="O1373" t="s">
         <v>424</v>
       </c>
@@ -66873,6 +67115,9 @@
       <c r="M1374">
         <v>5.31</v>
       </c>
+      <c r="N1374">
+        <v>1</v>
+      </c>
       <c r="O1374" t="s">
         <v>424</v>
       </c>
@@ -66923,6 +67168,9 @@
       <c r="M1375">
         <v>5.31</v>
       </c>
+      <c r="N1375">
+        <v>1</v>
+      </c>
       <c r="O1375" t="s">
         <v>424</v>
       </c>
@@ -66973,6 +67221,9 @@
       <c r="M1376">
         <v>5.31</v>
       </c>
+      <c r="N1376">
+        <v>1</v>
+      </c>
       <c r="O1376" t="s">
         <v>424</v>
       </c>
@@ -67175,6 +67426,9 @@
       <c r="M1381" s="9">
         <v>5.31</v>
       </c>
+      <c r="N1381" s="9">
+        <v>0</v>
+      </c>
       <c r="O1381" s="9" t="s">
         <v>425</v>
       </c>
@@ -67225,7 +67479,10 @@
       <c r="M1382" s="9">
         <v>5.31</v>
       </c>
-      <c r="O1382" s="18" t="s">
+      <c r="N1382" s="9">
+        <v>0</v>
+      </c>
+      <c r="O1382" t="s">
         <v>425</v>
       </c>
       <c r="P1382" s="9">
@@ -67275,7 +67532,10 @@
       <c r="M1383">
         <v>5.31</v>
       </c>
-      <c r="O1383" s="18" t="s">
+      <c r="N1383">
+        <v>1</v>
+      </c>
+      <c r="O1383" t="s">
         <v>425</v>
       </c>
       <c r="P1383">
@@ -67322,7 +67582,10 @@
       <c r="M1384">
         <v>5.31</v>
       </c>
-      <c r="O1384" s="18" t="s">
+      <c r="N1384">
+        <v>1</v>
+      </c>
+      <c r="O1384" t="s">
         <v>425</v>
       </c>
       <c r="P1384">
@@ -67369,7 +67632,10 @@
       <c r="M1385">
         <v>5.31</v>
       </c>
-      <c r="O1385" s="18" t="s">
+      <c r="N1385">
+        <v>1</v>
+      </c>
+      <c r="O1385" t="s">
         <v>425</v>
       </c>
       <c r="P1385">
@@ -67416,7 +67682,10 @@
       <c r="M1386" s="9">
         <v>5.31</v>
       </c>
-      <c r="O1386" s="18" t="s">
+      <c r="N1386" s="9">
+        <v>1</v>
+      </c>
+      <c r="O1386" t="s">
         <v>425</v>
       </c>
       <c r="P1386" s="9">
@@ -67463,7 +67732,10 @@
       <c r="M1387">
         <v>5.31</v>
       </c>
-      <c r="O1387" s="18" t="s">
+      <c r="N1387">
+        <v>1</v>
+      </c>
+      <c r="O1387" t="s">
         <v>425</v>
       </c>
       <c r="P1387">
@@ -67513,7 +67785,10 @@
       <c r="M1388">
         <v>5.31</v>
       </c>
-      <c r="O1388" s="18" t="s">
+      <c r="N1388">
+        <v>1</v>
+      </c>
+      <c r="O1388" t="s">
         <v>425</v>
       </c>
       <c r="P1388">
@@ -67563,7 +67838,10 @@
       <c r="M1389">
         <v>5.31</v>
       </c>
-      <c r="O1389" s="18" t="s">
+      <c r="N1389">
+        <v>1</v>
+      </c>
+      <c r="O1389" t="s">
         <v>425</v>
       </c>
       <c r="P1389">
@@ -67613,7 +67891,10 @@
       <c r="M1390">
         <v>5.31</v>
       </c>
-      <c r="O1390" s="18" t="s">
+      <c r="N1390">
+        <v>1</v>
+      </c>
+      <c r="O1390" t="s">
         <v>425</v>
       </c>
       <c r="P1390">
@@ -67660,7 +67941,10 @@
       <c r="M1391">
         <v>5.31</v>
       </c>
-      <c r="O1391" s="18" t="s">
+      <c r="N1391">
+        <v>1</v>
+      </c>
+      <c r="O1391" t="s">
         <v>425</v>
       </c>
       <c r="P1391">
@@ -67707,7 +67991,10 @@
       <c r="M1392">
         <v>5.31</v>
       </c>
-      <c r="O1392" s="18" t="s">
+      <c r="N1392">
+        <v>1</v>
+      </c>
+      <c r="O1392" t="s">
         <v>425</v>
       </c>
       <c r="P1392">
@@ -67754,7 +68041,10 @@
       <c r="M1393">
         <v>5.31</v>
       </c>
-      <c r="O1393" s="18" t="s">
+      <c r="N1393">
+        <v>1</v>
+      </c>
+      <c r="O1393" t="s">
         <v>425</v>
       </c>
       <c r="P1393">
@@ -67801,7 +68091,10 @@
       <c r="M1394">
         <v>5.31</v>
       </c>
-      <c r="O1394" s="18" t="s">
+      <c r="N1394">
+        <v>1</v>
+      </c>
+      <c r="O1394" t="s">
         <v>425</v>
       </c>
       <c r="P1394">
@@ -67848,7 +68141,10 @@
       <c r="M1395">
         <v>5.31</v>
       </c>
-      <c r="O1395" s="18" t="s">
+      <c r="N1395">
+        <v>1</v>
+      </c>
+      <c r="O1395" t="s">
         <v>425</v>
       </c>
       <c r="P1395">
@@ -67895,7 +68191,10 @@
       <c r="M1396">
         <v>5.31</v>
       </c>
-      <c r="O1396" s="18" t="s">
+      <c r="N1396">
+        <v>1</v>
+      </c>
+      <c r="O1396" t="s">
         <v>425</v>
       </c>
       <c r="P1396" s="5">
@@ -67945,7 +68244,10 @@
       <c r="M1397">
         <v>5.31</v>
       </c>
-      <c r="O1397" s="18" t="s">
+      <c r="N1397">
+        <v>1</v>
+      </c>
+      <c r="O1397" t="s">
         <v>425</v>
       </c>
       <c r="P1397">
@@ -67995,7 +68297,10 @@
       <c r="M1398">
         <v>5.31</v>
       </c>
-      <c r="O1398" s="18" t="s">
+      <c r="N1398">
+        <v>1</v>
+      </c>
+      <c r="O1398" t="s">
         <v>425</v>
       </c>
       <c r="P1398">
@@ -68045,7 +68350,10 @@
       <c r="M1399" s="9">
         <v>5.31</v>
       </c>
-      <c r="O1399" s="18" t="s">
+      <c r="N1399">
+        <v>1</v>
+      </c>
+      <c r="O1399" t="s">
         <v>425</v>
       </c>
       <c r="P1399" s="11">
@@ -68095,7 +68403,10 @@
       <c r="M1400">
         <v>5.31</v>
       </c>
-      <c r="O1400" s="18" t="s">
+      <c r="N1400">
+        <v>1</v>
+      </c>
+      <c r="O1400" t="s">
         <v>425</v>
       </c>
       <c r="P1400">
@@ -68145,7 +68456,10 @@
       <c r="M1401">
         <v>5.31</v>
       </c>
-      <c r="O1401" s="18" t="s">
+      <c r="N1401">
+        <v>1</v>
+      </c>
+      <c r="O1401" t="s">
         <v>425</v>
       </c>
       <c r="P1401">
@@ -68195,7 +68509,10 @@
       <c r="M1402">
         <v>5.31</v>
       </c>
-      <c r="O1402" s="18" t="s">
+      <c r="N1402">
+        <v>1</v>
+      </c>
+      <c r="O1402" t="s">
         <v>425</v>
       </c>
       <c r="P1402">
@@ -68242,7 +68559,10 @@
       <c r="M1403">
         <v>5.31</v>
       </c>
-      <c r="O1403" s="18" t="s">
+      <c r="N1403">
+        <v>1</v>
+      </c>
+      <c r="O1403" t="s">
         <v>425</v>
       </c>
       <c r="P1403" s="5">
@@ -68289,7 +68609,10 @@
       <c r="M1404">
         <v>5.31</v>
       </c>
-      <c r="O1404" s="18" t="s">
+      <c r="N1404">
+        <v>1</v>
+      </c>
+      <c r="O1404" t="s">
         <v>425</v>
       </c>
       <c r="P1404">
@@ -68336,7 +68659,10 @@
       <c r="M1405">
         <v>5.31</v>
       </c>
-      <c r="O1405" s="18" t="s">
+      <c r="N1405">
+        <v>1</v>
+      </c>
+      <c r="O1405" t="s">
         <v>425</v>
       </c>
       <c r="P1405">
@@ -68383,7 +68709,10 @@
       <c r="M1406">
         <v>5.31</v>
       </c>
-      <c r="O1406" s="18" t="s">
+      <c r="N1406">
+        <v>1</v>
+      </c>
+      <c r="O1406" t="s">
         <v>425</v>
       </c>
       <c r="P1406">
@@ -68430,7 +68759,10 @@
       <c r="M1407">
         <v>5.31</v>
       </c>
-      <c r="O1407" s="18" t="s">
+      <c r="N1407">
+        <v>1</v>
+      </c>
+      <c r="O1407" t="s">
         <v>425</v>
       </c>
       <c r="P1407">
@@ -68477,7 +68809,10 @@
       <c r="M1408">
         <v>5.31</v>
       </c>
-      <c r="O1408" s="18" t="s">
+      <c r="N1408">
+        <v>1</v>
+      </c>
+      <c r="O1408" t="s">
         <v>425</v>
       </c>
       <c r="P1408" s="8">
@@ -68524,7 +68859,10 @@
       <c r="M1409">
         <v>5.31</v>
       </c>
-      <c r="O1409" s="18" t="s">
+      <c r="N1409">
+        <v>1</v>
+      </c>
+      <c r="O1409" t="s">
         <v>425</v>
       </c>
       <c r="P1409" s="8">
@@ -68571,7 +68909,10 @@
       <c r="M1410">
         <v>5.31</v>
       </c>
-      <c r="O1410" s="18" t="s">
+      <c r="N1410">
+        <v>1</v>
+      </c>
+      <c r="O1410" t="s">
         <v>425</v>
       </c>
       <c r="P1410">
@@ -68618,7 +68959,10 @@
       <c r="M1411">
         <v>5.31</v>
       </c>
-      <c r="O1411" s="18" t="s">
+      <c r="N1411">
+        <v>1</v>
+      </c>
+      <c r="O1411" t="s">
         <v>425</v>
       </c>
       <c r="P1411">
@@ -68665,7 +69009,10 @@
       <c r="M1412">
         <v>5.31</v>
       </c>
-      <c r="O1412" s="18" t="s">
+      <c r="N1412">
+        <v>1</v>
+      </c>
+      <c r="O1412" t="s">
         <v>425</v>
       </c>
       <c r="P1412">
@@ -68712,7 +69059,10 @@
       <c r="M1413">
         <v>5.31</v>
       </c>
-      <c r="O1413" s="18" t="s">
+      <c r="N1413">
+        <v>1</v>
+      </c>
+      <c r="O1413" t="s">
         <v>425</v>
       </c>
       <c r="P1413" s="5">
@@ -68759,7 +69109,10 @@
       <c r="M1414">
         <v>5.31</v>
       </c>
-      <c r="O1414" s="18" t="s">
+      <c r="N1414">
+        <v>1</v>
+      </c>
+      <c r="O1414" t="s">
         <v>425</v>
       </c>
       <c r="P1414">
@@ -68806,7 +69159,10 @@
       <c r="M1415">
         <v>5.31</v>
       </c>
-      <c r="O1415" s="18" t="s">
+      <c r="N1415">
+        <v>1</v>
+      </c>
+      <c r="O1415" t="s">
         <v>425</v>
       </c>
       <c r="P1415" s="5">
@@ -68853,7 +69209,10 @@
       <c r="M1416">
         <v>5.31</v>
       </c>
-      <c r="O1416" s="18" t="s">
+      <c r="N1416">
+        <v>1</v>
+      </c>
+      <c r="O1416" t="s">
         <v>425</v>
       </c>
       <c r="P1416">
@@ -68900,7 +69259,10 @@
       <c r="M1417">
         <v>5.31</v>
       </c>
-      <c r="O1417" s="18" t="s">
+      <c r="N1417">
+        <v>1</v>
+      </c>
+      <c r="O1417" t="s">
         <v>425</v>
       </c>
       <c r="P1417">
@@ -68950,7 +69312,10 @@
       <c r="M1418" s="9">
         <v>5.31</v>
       </c>
-      <c r="O1418" s="18" t="s">
+      <c r="N1418" s="9">
+        <v>1</v>
+      </c>
+      <c r="O1418" t="s">
         <v>425</v>
       </c>
       <c r="P1418" s="9">
@@ -69000,7 +69365,10 @@
       <c r="M1419">
         <v>5.31</v>
       </c>
-      <c r="O1419" s="18" t="s">
+      <c r="N1419">
+        <v>1</v>
+      </c>
+      <c r="O1419" t="s">
         <v>425</v>
       </c>
       <c r="P1419">
@@ -69050,7 +69418,10 @@
       <c r="M1420">
         <v>5.31</v>
       </c>
-      <c r="O1420" s="18" t="s">
+      <c r="N1420">
+        <v>1</v>
+      </c>
+      <c r="O1420" t="s">
         <v>425</v>
       </c>
       <c r="P1420" s="5">
@@ -69097,7 +69468,10 @@
       <c r="M1421">
         <v>5.31</v>
       </c>
-      <c r="O1421" s="18" t="s">
+      <c r="N1421">
+        <v>1</v>
+      </c>
+      <c r="O1421" t="s">
         <v>425</v>
       </c>
       <c r="P1421">
@@ -69147,7 +69521,10 @@
       <c r="M1422">
         <v>5.31</v>
       </c>
-      <c r="O1422" s="18" t="s">
+      <c r="N1422">
+        <v>1</v>
+      </c>
+      <c r="O1422" t="s">
         <v>425</v>
       </c>
       <c r="P1422" s="5">
@@ -69185,6 +69562,9 @@
       <c r="M1423">
         <v>5.31</v>
       </c>
+      <c r="N1423">
+        <v>1</v>
+      </c>
     </row>
     <row r="1424" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A1424" t="s">
@@ -69217,6 +69597,9 @@
       <c r="M1424">
         <v>5.31</v>
       </c>
+      <c r="N1424">
+        <v>1</v>
+      </c>
     </row>
     <row r="1425" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A1425" t="s">
@@ -69249,6 +69632,9 @@
       <c r="M1425">
         <v>5.31</v>
       </c>
+      <c r="N1425">
+        <v>1</v>
+      </c>
     </row>
     <row r="1426" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A1426" t="s">
@@ -69281,6 +69667,9 @@
       <c r="M1426">
         <v>5.31</v>
       </c>
+      <c r="N1426">
+        <v>1</v>
+      </c>
     </row>
     <row r="1427" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A1427" t="s">
@@ -69322,6 +69711,9 @@
       <c r="M1427">
         <v>5.31</v>
       </c>
+      <c r="N1427">
+        <v>1</v>
+      </c>
       <c r="O1427" t="s">
         <v>316</v>
       </c>
@@ -69369,6 +69761,9 @@
       <c r="M1428">
         <v>5.31</v>
       </c>
+      <c r="N1428">
+        <v>1</v>
+      </c>
       <c r="O1428" t="s">
         <v>316</v>
       </c>
@@ -69416,6 +69811,9 @@
       <c r="M1429">
         <v>5.31</v>
       </c>
+      <c r="N1429">
+        <v>1</v>
+      </c>
       <c r="O1429" t="s">
         <v>316</v>
       </c>
@@ -69463,6 +69861,9 @@
       <c r="M1430">
         <v>5.31</v>
       </c>
+      <c r="N1430">
+        <v>1</v>
+      </c>
       <c r="O1430" t="s">
         <v>316</v>
       </c>
@@ -69510,6 +69911,9 @@
       <c r="M1431">
         <v>5.31</v>
       </c>
+      <c r="N1431">
+        <v>1</v>
+      </c>
       <c r="O1431" t="s">
         <v>316</v>
       </c>
@@ -69557,6 +69961,9 @@
       <c r="M1432" s="9">
         <v>5.31</v>
       </c>
+      <c r="N1432" s="9">
+        <v>1</v>
+      </c>
       <c r="O1432" s="9" t="s">
         <v>316</v>
       </c>
@@ -69607,6 +70014,9 @@
       <c r="M1433">
         <v>5.31</v>
       </c>
+      <c r="N1433">
+        <v>1</v>
+      </c>
       <c r="O1433" t="s">
         <v>316</v>
       </c>
@@ -69654,6 +70064,9 @@
       <c r="M1434">
         <v>5.31</v>
       </c>
+      <c r="N1434">
+        <v>1</v>
+      </c>
       <c r="O1434" t="s">
         <v>316</v>
       </c>
@@ -69701,6 +70114,9 @@
       <c r="M1435">
         <v>5.31</v>
       </c>
+      <c r="N1435">
+        <v>1</v>
+      </c>
       <c r="O1435" t="s">
         <v>316</v>
       </c>
@@ -69751,6 +70167,9 @@
       <c r="M1436">
         <v>5.31</v>
       </c>
+      <c r="N1436">
+        <v>1</v>
+      </c>
       <c r="O1436" t="s">
         <v>316</v>
       </c>
@@ -69798,6 +70217,9 @@
       <c r="M1437">
         <v>5.31</v>
       </c>
+      <c r="N1437">
+        <v>1</v>
+      </c>
       <c r="O1437" t="s">
         <v>316</v>
       </c>
@@ -69845,6 +70267,9 @@
       <c r="M1438">
         <v>5.31</v>
       </c>
+      <c r="N1438">
+        <v>1</v>
+      </c>
       <c r="O1438" t="s">
         <v>316</v>
       </c>
@@ -69892,6 +70317,9 @@
       <c r="M1439">
         <v>5.31</v>
       </c>
+      <c r="N1439">
+        <v>1</v>
+      </c>
       <c r="O1439" t="s">
         <v>316</v>
       </c>
@@ -69939,6 +70367,9 @@
       <c r="M1440">
         <v>5.31</v>
       </c>
+      <c r="N1440">
+        <v>1</v>
+      </c>
       <c r="O1440" t="s">
         <v>316</v>
       </c>
@@ -69986,6 +70417,9 @@
       <c r="M1441">
         <v>5.31</v>
       </c>
+      <c r="N1441">
+        <v>1</v>
+      </c>
       <c r="O1441" t="s">
         <v>316</v>
       </c>
@@ -70033,6 +70467,9 @@
       <c r="M1442">
         <v>5.31</v>
       </c>
+      <c r="N1442">
+        <v>1</v>
+      </c>
       <c r="O1442" t="s">
         <v>316</v>
       </c>
@@ -70080,6 +70517,9 @@
       <c r="M1443">
         <v>5.31</v>
       </c>
+      <c r="N1443">
+        <v>1</v>
+      </c>
       <c r="O1443" t="s">
         <v>316</v>
       </c>
@@ -70127,6 +70567,9 @@
       <c r="M1444">
         <v>5.31</v>
       </c>
+      <c r="N1444">
+        <v>1</v>
+      </c>
       <c r="O1444" t="s">
         <v>316</v>
       </c>
@@ -70174,6 +70617,9 @@
       <c r="M1445">
         <v>5.31</v>
       </c>
+      <c r="N1445">
+        <v>1</v>
+      </c>
       <c r="O1445" t="s">
         <v>316</v>
       </c>
@@ -70221,6 +70667,9 @@
       <c r="M1446">
         <v>5.31</v>
       </c>
+      <c r="N1446">
+        <v>1</v>
+      </c>
       <c r="O1446" t="s">
         <v>316</v>
       </c>
@@ -70268,6 +70717,9 @@
       <c r="M1447">
         <v>5.31</v>
       </c>
+      <c r="N1447">
+        <v>1</v>
+      </c>
       <c r="O1447" t="s">
         <v>316</v>
       </c>
@@ -70315,6 +70767,9 @@
       <c r="M1448">
         <v>5.31</v>
       </c>
+      <c r="N1448">
+        <v>1</v>
+      </c>
       <c r="O1448" t="s">
         <v>316</v>
       </c>
@@ -70362,6 +70817,9 @@
       <c r="M1449">
         <v>5.31</v>
       </c>
+      <c r="N1449">
+        <v>1</v>
+      </c>
       <c r="O1449" t="s">
         <v>316</v>
       </c>
@@ -70409,6 +70867,9 @@
       <c r="M1450">
         <v>5.31</v>
       </c>
+      <c r="N1450">
+        <v>1</v>
+      </c>
       <c r="O1450" t="s">
         <v>316</v>
       </c>
@@ -70456,6 +70917,9 @@
       <c r="M1451">
         <v>5.31</v>
       </c>
+      <c r="N1451">
+        <v>1</v>
+      </c>
       <c r="O1451" t="s">
         <v>316</v>
       </c>
@@ -70503,6 +70967,9 @@
       <c r="M1452">
         <v>5.31</v>
       </c>
+      <c r="N1452">
+        <v>1</v>
+      </c>
       <c r="O1452" t="s">
         <v>316</v>
       </c>
@@ -70550,6 +71017,9 @@
       <c r="M1453">
         <v>5.31</v>
       </c>
+      <c r="N1453">
+        <v>1</v>
+      </c>
       <c r="O1453" t="s">
         <v>316</v>
       </c>
@@ -70597,6 +71067,9 @@
       <c r="M1454">
         <v>5.31</v>
       </c>
+      <c r="N1454">
+        <v>1</v>
+      </c>
       <c r="O1454" t="s">
         <v>316</v>
       </c>
@@ -70644,6 +71117,9 @@
       <c r="M1455">
         <v>5.31</v>
       </c>
+      <c r="N1455">
+        <v>1</v>
+      </c>
       <c r="O1455" t="s">
         <v>316</v>
       </c>
@@ -70691,6 +71167,9 @@
       <c r="M1456">
         <v>5.31</v>
       </c>
+      <c r="N1456">
+        <v>1</v>
+      </c>
       <c r="O1456" t="s">
         <v>316</v>
       </c>
@@ -70738,6 +71217,9 @@
       <c r="M1457">
         <v>5.31</v>
       </c>
+      <c r="N1457">
+        <v>1</v>
+      </c>
       <c r="O1457" t="s">
         <v>316</v>
       </c>
@@ -70785,6 +71267,9 @@
       <c r="M1458">
         <v>5.31</v>
       </c>
+      <c r="N1458">
+        <v>1</v>
+      </c>
       <c r="O1458" t="s">
         <v>316</v>
       </c>
@@ -70832,6 +71317,9 @@
       <c r="M1459">
         <v>5.31</v>
       </c>
+      <c r="N1459">
+        <v>1</v>
+      </c>
       <c r="O1459" t="s">
         <v>316</v>
       </c>
@@ -70879,6 +71367,9 @@
       <c r="M1460">
         <v>5.31</v>
       </c>
+      <c r="N1460">
+        <v>1</v>
+      </c>
       <c r="O1460" t="s">
         <v>316</v>
       </c>
@@ -70926,6 +71417,9 @@
       <c r="M1461">
         <v>5.31</v>
       </c>
+      <c r="N1461">
+        <v>1</v>
+      </c>
       <c r="O1461" t="s">
         <v>316</v>
       </c>
@@ -70973,6 +71467,9 @@
       <c r="M1462">
         <v>5.31</v>
       </c>
+      <c r="N1462">
+        <v>1</v>
+      </c>
       <c r="O1462" t="s">
         <v>316</v>
       </c>
@@ -71020,6 +71517,9 @@
       <c r="M1463">
         <v>5.31</v>
       </c>
+      <c r="N1463">
+        <v>1</v>
+      </c>
       <c r="O1463" t="s">
         <v>316</v>
       </c>
@@ -71067,6 +71567,9 @@
       <c r="M1464">
         <v>5.31</v>
       </c>
+      <c r="N1464">
+        <v>1</v>
+      </c>
       <c r="O1464" t="s">
         <v>316</v>
       </c>
@@ -71114,6 +71617,9 @@
       <c r="M1465">
         <v>5.31</v>
       </c>
+      <c r="N1465">
+        <v>1</v>
+      </c>
       <c r="O1465" t="s">
         <v>316</v>
       </c>
@@ -71161,6 +71667,9 @@
       <c r="M1466">
         <v>5.31</v>
       </c>
+      <c r="N1466">
+        <v>1</v>
+      </c>
       <c r="O1466" t="s">
         <v>316</v>
       </c>
@@ -71208,6 +71717,9 @@
       <c r="M1467">
         <v>5.31</v>
       </c>
+      <c r="N1467">
+        <v>1</v>
+      </c>
       <c r="O1467" t="s">
         <v>316</v>
       </c>
@@ -71255,6 +71767,9 @@
       <c r="M1468">
         <v>5.31</v>
       </c>
+      <c r="N1468">
+        <v>1</v>
+      </c>
       <c r="O1468" t="s">
         <v>316</v>
       </c>
@@ -71418,6 +71933,9 @@
       <c r="M1473">
         <v>5.31</v>
       </c>
+      <c r="N1473">
+        <v>1</v>
+      </c>
       <c r="O1473" t="s">
         <v>317</v>
       </c>
@@ -71465,6 +71983,9 @@
       <c r="M1474">
         <v>5.31</v>
       </c>
+      <c r="N1474">
+        <v>1</v>
+      </c>
       <c r="O1474" t="s">
         <v>317</v>
       </c>
@@ -71512,6 +72033,9 @@
       <c r="M1475">
         <v>5.31</v>
       </c>
+      <c r="N1475">
+        <v>1</v>
+      </c>
       <c r="O1475" t="s">
         <v>317</v>
       </c>
@@ -71559,6 +72083,9 @@
       <c r="M1476">
         <v>5.31</v>
       </c>
+      <c r="N1476">
+        <v>1</v>
+      </c>
       <c r="O1476" t="s">
         <v>317</v>
       </c>
@@ -71606,6 +72133,9 @@
       <c r="M1477">
         <v>5.31</v>
       </c>
+      <c r="N1477">
+        <v>1</v>
+      </c>
       <c r="O1477" t="s">
         <v>317</v>
       </c>
@@ -71653,6 +72183,9 @@
       <c r="M1478">
         <v>5.31</v>
       </c>
+      <c r="N1478">
+        <v>1</v>
+      </c>
       <c r="O1478" t="s">
         <v>317</v>
       </c>
@@ -71700,6 +72233,9 @@
       <c r="M1479">
         <v>5.31</v>
       </c>
+      <c r="N1479">
+        <v>1</v>
+      </c>
       <c r="O1479" t="s">
         <v>317</v>
       </c>
@@ -71747,6 +72283,9 @@
       <c r="M1480">
         <v>5.31</v>
       </c>
+      <c r="N1480">
+        <v>1</v>
+      </c>
       <c r="O1480" t="s">
         <v>317</v>
       </c>
@@ -71794,6 +72333,9 @@
       <c r="M1481">
         <v>5.31</v>
       </c>
+      <c r="N1481">
+        <v>1</v>
+      </c>
       <c r="O1481" t="s">
         <v>317</v>
       </c>
@@ -71841,6 +72383,9 @@
       <c r="M1482">
         <v>5.31</v>
       </c>
+      <c r="N1482">
+        <v>1</v>
+      </c>
       <c r="O1482" t="s">
         <v>317</v>
       </c>
@@ -71888,6 +72433,9 @@
       <c r="M1483">
         <v>5.31</v>
       </c>
+      <c r="N1483">
+        <v>1</v>
+      </c>
       <c r="O1483" t="s">
         <v>317</v>
       </c>
@@ -71935,6 +72483,9 @@
       <c r="M1484">
         <v>5.31</v>
       </c>
+      <c r="N1484">
+        <v>1</v>
+      </c>
       <c r="O1484" t="s">
         <v>317</v>
       </c>
@@ -71982,6 +72533,9 @@
       <c r="M1485">
         <v>5.31</v>
       </c>
+      <c r="N1485">
+        <v>1</v>
+      </c>
       <c r="O1485" t="s">
         <v>317</v>
       </c>
@@ -72029,6 +72583,9 @@
       <c r="M1486">
         <v>5.31</v>
       </c>
+      <c r="N1486">
+        <v>1</v>
+      </c>
       <c r="O1486" t="s">
         <v>317</v>
       </c>
@@ -72076,6 +72633,9 @@
       <c r="M1487">
         <v>5.31</v>
       </c>
+      <c r="N1487">
+        <v>1</v>
+      </c>
       <c r="O1487" t="s">
         <v>317</v>
       </c>
@@ -72123,6 +72683,9 @@
       <c r="M1488">
         <v>5.31</v>
       </c>
+      <c r="N1488">
+        <v>1</v>
+      </c>
       <c r="O1488" t="s">
         <v>317</v>
       </c>
@@ -72170,6 +72733,9 @@
       <c r="M1489">
         <v>5.31</v>
       </c>
+      <c r="N1489">
+        <v>1</v>
+      </c>
       <c r="O1489" t="s">
         <v>317</v>
       </c>
@@ -72217,6 +72783,9 @@
       <c r="M1490">
         <v>5.31</v>
       </c>
+      <c r="N1490">
+        <v>1</v>
+      </c>
       <c r="O1490" t="s">
         <v>317</v>
       </c>
@@ -72264,6 +72833,9 @@
       <c r="M1491">
         <v>5.31</v>
       </c>
+      <c r="N1491">
+        <v>1</v>
+      </c>
       <c r="O1491" t="s">
         <v>317</v>
       </c>
@@ -72311,6 +72883,9 @@
       <c r="M1492">
         <v>5.31</v>
       </c>
+      <c r="N1492">
+        <v>1</v>
+      </c>
       <c r="O1492" t="s">
         <v>317</v>
       </c>
@@ -72358,6 +72933,9 @@
       <c r="M1493">
         <v>5.31</v>
       </c>
+      <c r="N1493">
+        <v>1</v>
+      </c>
       <c r="O1493" t="s">
         <v>317</v>
       </c>
@@ -72405,6 +72983,9 @@
       <c r="M1494">
         <v>5.31</v>
       </c>
+      <c r="N1494">
+        <v>1</v>
+      </c>
       <c r="O1494" t="s">
         <v>317</v>
       </c>
@@ -72452,6 +73033,9 @@
       <c r="M1495">
         <v>5.31</v>
       </c>
+      <c r="N1495">
+        <v>1</v>
+      </c>
       <c r="O1495" t="s">
         <v>317</v>
       </c>
@@ -72499,6 +73083,9 @@
       <c r="M1496">
         <v>5.31</v>
       </c>
+      <c r="N1496">
+        <v>1</v>
+      </c>
       <c r="O1496" t="s">
         <v>317</v>
       </c>
@@ -72546,6 +73133,9 @@
       <c r="M1497">
         <v>5.31</v>
       </c>
+      <c r="N1497">
+        <v>1</v>
+      </c>
       <c r="O1497" t="s">
         <v>317</v>
       </c>
@@ -72593,6 +73183,9 @@
       <c r="M1498">
         <v>5.31</v>
       </c>
+      <c r="N1498">
+        <v>1</v>
+      </c>
       <c r="O1498" t="s">
         <v>317</v>
       </c>
@@ -72640,6 +73233,9 @@
       <c r="M1499">
         <v>5.31</v>
       </c>
+      <c r="N1499">
+        <v>1</v>
+      </c>
       <c r="O1499" t="s">
         <v>317</v>
       </c>
@@ -72687,6 +73283,9 @@
       <c r="M1500">
         <v>5.31</v>
       </c>
+      <c r="N1500">
+        <v>1</v>
+      </c>
       <c r="O1500" t="s">
         <v>317</v>
       </c>
@@ -72734,6 +73333,9 @@
       <c r="M1501">
         <v>5.31</v>
       </c>
+      <c r="N1501">
+        <v>1</v>
+      </c>
       <c r="O1501" t="s">
         <v>317</v>
       </c>
@@ -72781,6 +73383,9 @@
       <c r="M1502">
         <v>5.31</v>
       </c>
+      <c r="N1502">
+        <v>1</v>
+      </c>
       <c r="O1502" t="s">
         <v>317</v>
       </c>
@@ -72828,6 +73433,9 @@
       <c r="M1503">
         <v>5.31</v>
       </c>
+      <c r="N1503">
+        <v>1</v>
+      </c>
       <c r="O1503" t="s">
         <v>317</v>
       </c>
@@ -72875,6 +73483,9 @@
       <c r="M1504">
         <v>5.31</v>
       </c>
+      <c r="N1504">
+        <v>1</v>
+      </c>
       <c r="O1504" t="s">
         <v>317</v>
       </c>
@@ -72922,6 +73533,9 @@
       <c r="M1505">
         <v>5.31</v>
       </c>
+      <c r="N1505">
+        <v>1</v>
+      </c>
       <c r="O1505" t="s">
         <v>317</v>
       </c>
@@ -72969,6 +73583,9 @@
       <c r="M1506">
         <v>5.31</v>
       </c>
+      <c r="N1506">
+        <v>1</v>
+      </c>
       <c r="O1506" t="s">
         <v>317</v>
       </c>
@@ -73016,6 +73633,9 @@
       <c r="M1507">
         <v>5.31</v>
       </c>
+      <c r="N1507">
+        <v>1</v>
+      </c>
       <c r="O1507" t="s">
         <v>317</v>
       </c>
@@ -73063,6 +73683,9 @@
       <c r="M1508">
         <v>5.31</v>
       </c>
+      <c r="N1508">
+        <v>1</v>
+      </c>
       <c r="O1508" t="s">
         <v>317</v>
       </c>
@@ -73110,6 +73733,9 @@
       <c r="M1509">
         <v>5.31</v>
       </c>
+      <c r="N1509">
+        <v>1</v>
+      </c>
       <c r="O1509" t="s">
         <v>317</v>
       </c>
@@ -73157,6 +73783,9 @@
       <c r="M1510">
         <v>5.31</v>
       </c>
+      <c r="N1510">
+        <v>1</v>
+      </c>
       <c r="O1510" t="s">
         <v>317</v>
       </c>
@@ -73204,6 +73833,9 @@
       <c r="M1511">
         <v>5.31</v>
       </c>
+      <c r="N1511">
+        <v>1</v>
+      </c>
       <c r="O1511" t="s">
         <v>317</v>
       </c>
@@ -73251,6 +73883,9 @@
       <c r="M1512">
         <v>5.31</v>
       </c>
+      <c r="N1512">
+        <v>1</v>
+      </c>
       <c r="O1512" t="s">
         <v>317</v>
       </c>
@@ -73298,6 +73933,9 @@
       <c r="M1513">
         <v>5.31</v>
       </c>
+      <c r="N1513">
+        <v>1</v>
+      </c>
       <c r="O1513" t="s">
         <v>317</v>
       </c>
@@ -73345,6 +73983,9 @@
       <c r="M1514">
         <v>5.31</v>
       </c>
+      <c r="N1514">
+        <v>1</v>
+      </c>
       <c r="O1514" t="s">
         <v>317</v>
       </c>
@@ -73508,6 +74149,9 @@
       <c r="M1519">
         <v>5.31</v>
       </c>
+      <c r="N1519">
+        <v>1</v>
+      </c>
       <c r="O1519" t="s">
         <v>318</v>
       </c>
@@ -73555,6 +74199,9 @@
       <c r="M1520">
         <v>5.31</v>
       </c>
+      <c r="N1520">
+        <v>1</v>
+      </c>
       <c r="O1520" t="s">
         <v>318</v>
       </c>
@@ -73602,6 +74249,9 @@
       <c r="M1521">
         <v>5.31</v>
       </c>
+      <c r="N1521">
+        <v>1</v>
+      </c>
       <c r="O1521" t="s">
         <v>318</v>
       </c>
@@ -73649,6 +74299,9 @@
       <c r="M1522">
         <v>5.31</v>
       </c>
+      <c r="N1522">
+        <v>1</v>
+      </c>
       <c r="O1522" t="s">
         <v>318</v>
       </c>
@@ -73696,6 +74349,9 @@
       <c r="M1523">
         <v>5.31</v>
       </c>
+      <c r="N1523">
+        <v>1</v>
+      </c>
       <c r="O1523" t="s">
         <v>318</v>
       </c>
@@ -73743,6 +74399,9 @@
       <c r="M1524">
         <v>5.31</v>
       </c>
+      <c r="N1524">
+        <v>1</v>
+      </c>
       <c r="O1524" t="s">
         <v>318</v>
       </c>
@@ -73790,6 +74449,9 @@
       <c r="M1525">
         <v>5.31</v>
       </c>
+      <c r="N1525">
+        <v>1</v>
+      </c>
       <c r="O1525" t="s">
         <v>318</v>
       </c>
@@ -73837,6 +74499,9 @@
       <c r="M1526">
         <v>5.31</v>
       </c>
+      <c r="N1526">
+        <v>1</v>
+      </c>
       <c r="O1526" t="s">
         <v>318</v>
       </c>
@@ -73884,6 +74549,9 @@
       <c r="M1527">
         <v>5.31</v>
       </c>
+      <c r="N1527">
+        <v>1</v>
+      </c>
       <c r="O1527" t="s">
         <v>318</v>
       </c>
@@ -73932,6 +74600,9 @@
         <f>5.31/2</f>
         <v>2.6549999999999998</v>
       </c>
+      <c r="N1528">
+        <v>1</v>
+      </c>
       <c r="O1528" t="s">
         <v>318</v>
       </c>
@@ -73982,6 +74653,9 @@
       <c r="M1529">
         <v>5.31</v>
       </c>
+      <c r="N1529">
+        <v>1</v>
+      </c>
       <c r="O1529" t="s">
         <v>318</v>
       </c>
@@ -74029,6 +74703,9 @@
       <c r="M1530">
         <v>5.31</v>
       </c>
+      <c r="N1530">
+        <v>1</v>
+      </c>
       <c r="O1530" t="s">
         <v>318</v>
       </c>
@@ -74079,6 +74756,9 @@
       <c r="M1531">
         <v>5.31</v>
       </c>
+      <c r="N1531">
+        <v>1</v>
+      </c>
       <c r="O1531" t="s">
         <v>318</v>
       </c>
@@ -74129,6 +74809,9 @@
       <c r="M1532">
         <v>5.31</v>
       </c>
+      <c r="N1532">
+        <v>1</v>
+      </c>
       <c r="O1532" t="s">
         <v>318</v>
       </c>
@@ -74176,6 +74859,9 @@
       <c r="M1533">
         <v>5.31</v>
       </c>
+      <c r="N1533">
+        <v>1</v>
+      </c>
       <c r="O1533" t="s">
         <v>318</v>
       </c>
@@ -74223,6 +74909,9 @@
       <c r="M1534">
         <v>5.31</v>
       </c>
+      <c r="N1534">
+        <v>1</v>
+      </c>
       <c r="O1534" t="s">
         <v>318</v>
       </c>
@@ -74270,6 +74959,9 @@
       <c r="M1535">
         <v>5.31</v>
       </c>
+      <c r="N1535">
+        <v>1</v>
+      </c>
       <c r="O1535" t="s">
         <v>318</v>
       </c>
@@ -74317,6 +75009,9 @@
       <c r="M1536">
         <v>5.31</v>
       </c>
+      <c r="N1536">
+        <v>1</v>
+      </c>
       <c r="O1536" t="s">
         <v>318</v>
       </c>
@@ -74364,6 +75059,9 @@
       <c r="M1537">
         <v>5.31</v>
       </c>
+      <c r="N1537">
+        <v>1</v>
+      </c>
       <c r="O1537" t="s">
         <v>318</v>
       </c>
@@ -74414,6 +75112,9 @@
       <c r="M1538" s="9">
         <v>5.31</v>
       </c>
+      <c r="N1538">
+        <v>1</v>
+      </c>
       <c r="O1538" s="9" t="s">
         <v>318</v>
       </c>
@@ -74464,6 +75165,9 @@
       <c r="M1539">
         <v>5.31</v>
       </c>
+      <c r="N1539">
+        <v>1</v>
+      </c>
       <c r="O1539" t="s">
         <v>318</v>
       </c>
@@ -74514,6 +75218,9 @@
       <c r="M1540">
         <v>5.31</v>
       </c>
+      <c r="N1540">
+        <v>1</v>
+      </c>
       <c r="O1540" t="s">
         <v>318</v>
       </c>
@@ -74561,6 +75268,9 @@
       <c r="M1541">
         <v>5.31</v>
       </c>
+      <c r="N1541">
+        <v>1</v>
+      </c>
       <c r="O1541" t="s">
         <v>318</v>
       </c>
@@ -74608,6 +75318,9 @@
       <c r="M1542">
         <v>5.31</v>
       </c>
+      <c r="N1542">
+        <v>1</v>
+      </c>
       <c r="O1542" t="s">
         <v>318</v>
       </c>
@@ -74655,6 +75368,9 @@
       <c r="M1543">
         <v>5.31</v>
       </c>
+      <c r="N1543">
+        <v>1</v>
+      </c>
       <c r="O1543" t="s">
         <v>318</v>
       </c>
@@ -74702,6 +75418,9 @@
       <c r="M1544">
         <v>5.31</v>
       </c>
+      <c r="N1544">
+        <v>1</v>
+      </c>
       <c r="O1544" t="s">
         <v>318</v>
       </c>
@@ -74749,6 +75468,9 @@
       <c r="M1545">
         <v>5.31</v>
       </c>
+      <c r="N1545">
+        <v>1</v>
+      </c>
       <c r="O1545" t="s">
         <v>318</v>
       </c>
@@ -74796,6 +75518,9 @@
       <c r="M1546">
         <v>5.31</v>
       </c>
+      <c r="N1546">
+        <v>1</v>
+      </c>
       <c r="O1546" t="s">
         <v>318</v>
       </c>
@@ -74843,6 +75568,9 @@
       <c r="M1547">
         <v>5.31</v>
       </c>
+      <c r="N1547">
+        <v>1</v>
+      </c>
       <c r="O1547" t="s">
         <v>318</v>
       </c>
@@ -74890,6 +75618,9 @@
       <c r="M1548">
         <v>5.31</v>
       </c>
+      <c r="N1548">
+        <v>1</v>
+      </c>
       <c r="O1548" t="s">
         <v>318</v>
       </c>
@@ -74937,6 +75668,9 @@
       <c r="M1549">
         <v>5.31</v>
       </c>
+      <c r="N1549">
+        <v>1</v>
+      </c>
       <c r="O1549" t="s">
         <v>318</v>
       </c>
@@ -74984,6 +75718,9 @@
       <c r="M1550">
         <v>5.31</v>
       </c>
+      <c r="N1550">
+        <v>1</v>
+      </c>
       <c r="O1550" t="s">
         <v>318</v>
       </c>
@@ -75031,6 +75768,9 @@
       <c r="M1551">
         <v>5.31</v>
       </c>
+      <c r="N1551">
+        <v>1</v>
+      </c>
       <c r="O1551" t="s">
         <v>318</v>
       </c>
@@ -75078,6 +75818,9 @@
       <c r="M1552">
         <v>5.31</v>
       </c>
+      <c r="N1552">
+        <v>1</v>
+      </c>
       <c r="O1552" t="s">
         <v>318</v>
       </c>
@@ -75125,6 +75868,9 @@
       <c r="M1553">
         <v>5.31</v>
       </c>
+      <c r="N1553">
+        <v>1</v>
+      </c>
       <c r="O1553" t="s">
         <v>318</v>
       </c>
@@ -75225,6 +75971,9 @@
       <c r="M1555">
         <v>5.31</v>
       </c>
+      <c r="N1555">
+        <v>1</v>
+      </c>
       <c r="O1555" t="s">
         <v>318</v>
       </c>
@@ -75272,6 +76021,9 @@
       <c r="M1556">
         <v>5.31</v>
       </c>
+      <c r="N1556">
+        <v>1</v>
+      </c>
       <c r="O1556" t="s">
         <v>318</v>
       </c>
@@ -75319,6 +76071,9 @@
       <c r="M1557">
         <v>5.31</v>
       </c>
+      <c r="N1557">
+        <v>1</v>
+      </c>
       <c r="O1557" t="s">
         <v>318</v>
       </c>
@@ -75366,6 +76121,9 @@
       <c r="M1558">
         <v>5.31</v>
       </c>
+      <c r="N1558">
+        <v>1</v>
+      </c>
       <c r="O1558" t="s">
         <v>318</v>
       </c>
@@ -75413,6 +76171,9 @@
       <c r="M1559">
         <v>5.31</v>
       </c>
+      <c r="N1559">
+        <v>1</v>
+      </c>
       <c r="O1559" t="s">
         <v>318</v>
       </c>
@@ -75460,6 +76221,9 @@
       <c r="M1560">
         <v>5.31</v>
       </c>
+      <c r="N1560">
+        <v>1</v>
+      </c>
       <c r="O1560" t="s">
         <v>318</v>
       </c>
@@ -75635,6 +76399,9 @@
       <c r="M1565">
         <v>5.31</v>
       </c>
+      <c r="N1565">
+        <v>1</v>
+      </c>
       <c r="O1565" t="s">
         <v>319</v>
       </c>
@@ -75685,6 +76452,9 @@
       <c r="M1566">
         <v>5.31</v>
       </c>
+      <c r="N1566">
+        <v>1</v>
+      </c>
       <c r="O1566" t="s">
         <v>319</v>
       </c>
@@ -75735,6 +76505,9 @@
       <c r="M1567">
         <v>5.31</v>
       </c>
+      <c r="N1567">
+        <v>1</v>
+      </c>
       <c r="O1567" t="s">
         <v>319</v>
       </c>
@@ -75785,6 +76558,9 @@
       <c r="M1568">
         <v>5.31</v>
       </c>
+      <c r="N1568">
+        <v>1</v>
+      </c>
       <c r="O1568" t="s">
         <v>319</v>
       </c>
@@ -75835,6 +76611,9 @@
       <c r="M1569">
         <v>5.31</v>
       </c>
+      <c r="N1569">
+        <v>1</v>
+      </c>
       <c r="O1569" t="s">
         <v>319</v>
       </c>
@@ -75885,6 +76664,9 @@
       <c r="M1570">
         <v>5.31</v>
       </c>
+      <c r="N1570">
+        <v>1</v>
+      </c>
       <c r="O1570" t="s">
         <v>319</v>
       </c>
@@ -75936,6 +76718,9 @@
       <c r="M1571">
         <v>5.31</v>
       </c>
+      <c r="N1571">
+        <v>1</v>
+      </c>
       <c r="O1571" t="s">
         <v>319</v>
       </c>
@@ -75986,6 +76771,9 @@
       <c r="M1572">
         <v>5.31</v>
       </c>
+      <c r="N1572">
+        <v>1</v>
+      </c>
       <c r="O1572" t="s">
         <v>319</v>
       </c>
@@ -76036,6 +76824,9 @@
       <c r="M1573">
         <v>5.31</v>
       </c>
+      <c r="N1573">
+        <v>1</v>
+      </c>
       <c r="O1573" t="s">
         <v>319</v>
       </c>
@@ -76086,6 +76877,9 @@
       <c r="M1574">
         <v>5.31</v>
       </c>
+      <c r="N1574">
+        <v>1</v>
+      </c>
       <c r="O1574" t="s">
         <v>319</v>
       </c>
@@ -76136,6 +76930,9 @@
       <c r="M1575">
         <v>5.31</v>
       </c>
+      <c r="N1575">
+        <v>1</v>
+      </c>
       <c r="O1575" t="s">
         <v>319</v>
       </c>
@@ -76186,6 +76983,9 @@
       <c r="M1576">
         <v>5.31</v>
       </c>
+      <c r="N1576">
+        <v>1</v>
+      </c>
       <c r="O1576" t="s">
         <v>319</v>
       </c>
@@ -76236,6 +77036,9 @@
       <c r="M1577">
         <v>5.31</v>
       </c>
+      <c r="N1577">
+        <v>1</v>
+      </c>
       <c r="O1577" t="s">
         <v>319</v>
       </c>
@@ -76287,6 +77090,9 @@
       <c r="M1578">
         <v>5.31</v>
       </c>
+      <c r="N1578">
+        <v>1</v>
+      </c>
       <c r="O1578" t="s">
         <v>319</v>
       </c>
@@ -76337,6 +77143,9 @@
       <c r="M1579">
         <v>5.31</v>
       </c>
+      <c r="N1579">
+        <v>1</v>
+      </c>
       <c r="O1579" t="s">
         <v>319</v>
       </c>
@@ -76387,6 +77196,9 @@
       <c r="M1580">
         <v>5.31</v>
       </c>
+      <c r="N1580">
+        <v>1</v>
+      </c>
       <c r="O1580" t="s">
         <v>319</v>
       </c>
@@ -76438,6 +77250,9 @@
       <c r="M1581">
         <v>5.31</v>
       </c>
+      <c r="N1581">
+        <v>1</v>
+      </c>
       <c r="O1581" t="s">
         <v>319</v>
       </c>
@@ -76488,6 +77303,9 @@
       <c r="M1582">
         <v>5.31</v>
       </c>
+      <c r="N1582">
+        <v>1</v>
+      </c>
       <c r="O1582" t="s">
         <v>319</v>
       </c>
@@ -76538,6 +77356,9 @@
       <c r="M1583">
         <v>5.31</v>
       </c>
+      <c r="N1583">
+        <v>1</v>
+      </c>
       <c r="O1583" t="s">
         <v>319</v>
       </c>
@@ -76588,6 +77409,9 @@
       <c r="M1584">
         <v>5.31</v>
       </c>
+      <c r="N1584">
+        <v>1</v>
+      </c>
       <c r="O1584" t="s">
         <v>319</v>
       </c>
@@ -76639,6 +77463,9 @@
       <c r="M1585">
         <v>5.31</v>
       </c>
+      <c r="N1585">
+        <v>1</v>
+      </c>
       <c r="O1585" t="s">
         <v>319</v>
       </c>
@@ -76689,6 +77516,9 @@
       <c r="M1586">
         <v>5.31</v>
       </c>
+      <c r="N1586">
+        <v>1</v>
+      </c>
       <c r="O1586" t="s">
         <v>319</v>
       </c>
@@ -76739,6 +77569,9 @@
       <c r="M1587">
         <v>5.31</v>
       </c>
+      <c r="N1587">
+        <v>1</v>
+      </c>
       <c r="O1587" t="s">
         <v>319</v>
       </c>
@@ -76789,6 +77622,9 @@
       <c r="M1588">
         <v>5.31</v>
       </c>
+      <c r="N1588">
+        <v>1</v>
+      </c>
       <c r="O1588" t="s">
         <v>319</v>
       </c>
@@ -76839,6 +77675,9 @@
       <c r="M1589">
         <v>5.31</v>
       </c>
+      <c r="N1589">
+        <v>1</v>
+      </c>
       <c r="O1589" t="s">
         <v>319</v>
       </c>
@@ -76889,6 +77728,9 @@
       <c r="M1590">
         <v>5.31</v>
       </c>
+      <c r="N1590">
+        <v>1</v>
+      </c>
       <c r="O1590" t="s">
         <v>319</v>
       </c>
@@ -76939,6 +77781,9 @@
       <c r="M1591">
         <v>5.31</v>
       </c>
+      <c r="N1591">
+        <v>1</v>
+      </c>
       <c r="O1591" t="s">
         <v>319</v>
       </c>
@@ -76989,6 +77834,9 @@
       <c r="M1592">
         <v>5.31</v>
       </c>
+      <c r="N1592">
+        <v>1</v>
+      </c>
       <c r="O1592" t="s">
         <v>319</v>
       </c>
@@ -77039,6 +77887,9 @@
       <c r="M1593">
         <v>5.31</v>
       </c>
+      <c r="N1593">
+        <v>1</v>
+      </c>
       <c r="O1593" t="s">
         <v>319</v>
       </c>
@@ -77089,6 +77940,9 @@
       <c r="M1594">
         <v>5.31</v>
       </c>
+      <c r="N1594">
+        <v>1</v>
+      </c>
       <c r="O1594" t="s">
         <v>319</v>
       </c>
@@ -77139,6 +77993,9 @@
       <c r="M1595">
         <v>5.31</v>
       </c>
+      <c r="N1595">
+        <v>1</v>
+      </c>
       <c r="O1595" t="s">
         <v>319</v>
       </c>
@@ -77190,6 +78047,9 @@
         <f>(5.31/4)*3</f>
         <v>3.9824999999999999</v>
       </c>
+      <c r="N1596">
+        <v>1</v>
+      </c>
       <c r="O1596" t="s">
         <v>319</v>
       </c>
@@ -77241,6 +78101,9 @@
         <f>(5.31/4)*3</f>
         <v>3.9824999999999999</v>
       </c>
+      <c r="N1597">
+        <v>1</v>
+      </c>
       <c r="O1597" t="s">
         <v>319</v>
       </c>
@@ -77291,6 +78154,9 @@
       <c r="M1598">
         <v>5.31</v>
       </c>
+      <c r="N1598">
+        <v>1</v>
+      </c>
       <c r="O1598" t="s">
         <v>319</v>
       </c>
@@ -77341,6 +78207,9 @@
       <c r="M1599">
         <v>5.31</v>
       </c>
+      <c r="N1599">
+        <v>1</v>
+      </c>
       <c r="O1599" t="s">
         <v>319</v>
       </c>
@@ -77391,6 +78260,9 @@
       <c r="M1600">
         <v>5.31</v>
       </c>
+      <c r="N1600">
+        <v>1</v>
+      </c>
       <c r="O1600" t="s">
         <v>319</v>
       </c>
@@ -77441,6 +78313,9 @@
       <c r="M1601">
         <v>5.31</v>
       </c>
+      <c r="N1601">
+        <v>1</v>
+      </c>
       <c r="O1601" t="s">
         <v>319</v>
       </c>
@@ -77491,6 +78366,9 @@
       <c r="M1602">
         <v>5.31</v>
       </c>
+      <c r="N1602">
+        <v>1</v>
+      </c>
       <c r="O1602" t="s">
         <v>319</v>
       </c>
@@ -77541,6 +78419,9 @@
       <c r="M1603">
         <v>5.31</v>
       </c>
+      <c r="N1603">
+        <v>1</v>
+      </c>
       <c r="O1603" t="s">
         <v>319</v>
       </c>
@@ -77591,6 +78472,9 @@
       <c r="M1604">
         <v>5.31</v>
       </c>
+      <c r="N1604">
+        <v>1</v>
+      </c>
       <c r="O1604" t="s">
         <v>319</v>
       </c>
@@ -77641,6 +78525,9 @@
       <c r="M1605">
         <v>5.31</v>
       </c>
+      <c r="N1605">
+        <v>1</v>
+      </c>
       <c r="O1605" t="s">
         <v>319</v>
       </c>
@@ -77691,6 +78578,9 @@
       <c r="M1606">
         <v>5.31</v>
       </c>
+      <c r="N1606">
+        <v>1</v>
+      </c>
       <c r="O1606" t="s">
         <v>319</v>
       </c>
@@ -77866,6 +78756,9 @@
       <c r="M1611">
         <v>5.31</v>
       </c>
+      <c r="N1611">
+        <v>1</v>
+      </c>
       <c r="O1611" t="s">
         <v>426</v>
       </c>
@@ -77913,6 +78806,9 @@
       <c r="M1612">
         <v>5.31</v>
       </c>
+      <c r="N1612">
+        <v>1</v>
+      </c>
       <c r="O1612" t="s">
         <v>426</v>
       </c>
@@ -77960,6 +78856,9 @@
       <c r="M1613">
         <v>5.31</v>
       </c>
+      <c r="N1613">
+        <v>1</v>
+      </c>
       <c r="O1613" t="s">
         <v>426</v>
       </c>
@@ -78007,6 +78906,9 @@
       <c r="M1614">
         <v>5.31</v>
       </c>
+      <c r="N1614">
+        <v>1</v>
+      </c>
       <c r="O1614" t="s">
         <v>426</v>
       </c>
@@ -78054,6 +78956,9 @@
       <c r="M1615">
         <v>5.31</v>
       </c>
+      <c r="N1615">
+        <v>1</v>
+      </c>
       <c r="O1615" t="s">
         <v>426</v>
       </c>
@@ -78101,6 +79006,9 @@
       <c r="M1616">
         <v>5.31</v>
       </c>
+      <c r="N1616">
+        <v>1</v>
+      </c>
       <c r="O1616" t="s">
         <v>426</v>
       </c>
@@ -78148,6 +79056,9 @@
       <c r="M1617">
         <v>5.31</v>
       </c>
+      <c r="N1617">
+        <v>1</v>
+      </c>
       <c r="O1617" t="s">
         <v>426</v>
       </c>
@@ -78192,6 +79103,9 @@
       <c r="M1618">
         <v>5.31</v>
       </c>
+      <c r="N1618">
+        <v>1</v>
+      </c>
       <c r="O1618" t="s">
         <v>426</v>
       </c>
@@ -78236,6 +79150,9 @@
       <c r="M1619">
         <v>5.31</v>
       </c>
+      <c r="N1619">
+        <v>1</v>
+      </c>
       <c r="O1619" t="s">
         <v>426</v>
       </c>
@@ -78280,6 +79197,9 @@
       <c r="M1620">
         <v>5.31</v>
       </c>
+      <c r="N1620">
+        <v>1</v>
+      </c>
       <c r="O1620" t="s">
         <v>426</v>
       </c>
@@ -78324,6 +79244,9 @@
       <c r="M1621">
         <v>5.31</v>
       </c>
+      <c r="N1621">
+        <v>1</v>
+      </c>
       <c r="O1621" t="s">
         <v>426</v>
       </c>
@@ -78368,6 +79291,9 @@
       <c r="M1622">
         <v>5.31</v>
       </c>
+      <c r="N1622">
+        <v>1</v>
+      </c>
       <c r="O1622" t="s">
         <v>426</v>
       </c>
@@ -78412,6 +79338,9 @@
       <c r="M1623">
         <v>5.31</v>
       </c>
+      <c r="N1623">
+        <v>1</v>
+      </c>
       <c r="O1623" t="s">
         <v>426</v>
       </c>
@@ -78456,6 +79385,9 @@
       <c r="M1624">
         <v>5.31</v>
       </c>
+      <c r="N1624">
+        <v>1</v>
+      </c>
       <c r="O1624" t="s">
         <v>426</v>
       </c>
@@ -78500,6 +79432,9 @@
       <c r="M1625">
         <v>5.31</v>
       </c>
+      <c r="N1625">
+        <v>1</v>
+      </c>
       <c r="O1625" t="s">
         <v>426</v>
       </c>
@@ -78544,6 +79479,9 @@
       <c r="M1626">
         <v>5.31</v>
       </c>
+      <c r="N1626">
+        <v>1</v>
+      </c>
       <c r="O1626" t="s">
         <v>426</v>
       </c>
@@ -78588,6 +79526,9 @@
       <c r="M1627">
         <v>5.31</v>
       </c>
+      <c r="N1627">
+        <v>1</v>
+      </c>
       <c r="O1627" t="s">
         <v>426</v>
       </c>
@@ -78632,6 +79573,9 @@
       <c r="M1628">
         <v>5.31</v>
       </c>
+      <c r="N1628">
+        <v>1</v>
+      </c>
       <c r="O1628" t="s">
         <v>426</v>
       </c>
@@ -78676,6 +79620,9 @@
       <c r="M1629">
         <v>5.31</v>
       </c>
+      <c r="N1629">
+        <v>1</v>
+      </c>
       <c r="O1629" t="s">
         <v>426</v>
       </c>
@@ -78720,6 +79667,9 @@
       <c r="M1630">
         <v>5.31</v>
       </c>
+      <c r="N1630">
+        <v>1</v>
+      </c>
       <c r="O1630" t="s">
         <v>426</v>
       </c>
@@ -78764,6 +79714,9 @@
       <c r="M1631">
         <v>5.31</v>
       </c>
+      <c r="N1631">
+        <v>1</v>
+      </c>
       <c r="O1631" t="s">
         <v>426</v>
       </c>
@@ -78808,6 +79761,9 @@
       <c r="M1632">
         <v>5.31</v>
       </c>
+      <c r="N1632">
+        <v>1</v>
+      </c>
       <c r="O1632" t="s">
         <v>426</v>
       </c>
@@ -78855,6 +79811,9 @@
       <c r="M1633">
         <v>5.31</v>
       </c>
+      <c r="N1633">
+        <v>1</v>
+      </c>
       <c r="O1633" t="s">
         <v>426</v>
       </c>
@@ -78902,6 +79861,9 @@
       <c r="M1634">
         <v>5.31</v>
       </c>
+      <c r="N1634">
+        <v>1</v>
+      </c>
       <c r="O1634" t="s">
         <v>426</v>
       </c>
@@ -78949,6 +79911,9 @@
       <c r="M1635">
         <v>5.31</v>
       </c>
+      <c r="N1635">
+        <v>1</v>
+      </c>
       <c r="O1635" t="s">
         <v>426</v>
       </c>
@@ -78996,6 +79961,9 @@
       <c r="M1636">
         <v>5.31</v>
       </c>
+      <c r="N1636">
+        <v>1</v>
+      </c>
       <c r="O1636" t="s">
         <v>426</v>
       </c>
@@ -79043,6 +80011,9 @@
       <c r="M1637" s="9">
         <v>5.31</v>
       </c>
+      <c r="N1637" s="9">
+        <v>0</v>
+      </c>
       <c r="O1637" t="s">
         <v>426</v>
       </c>
@@ -79090,6 +80061,9 @@
       <c r="M1638">
         <v>5.31</v>
       </c>
+      <c r="N1638">
+        <v>1</v>
+      </c>
       <c r="O1638" t="s">
         <v>426</v>
       </c>
@@ -79134,6 +80108,9 @@
       <c r="M1639">
         <v>5.31</v>
       </c>
+      <c r="N1639">
+        <v>1</v>
+      </c>
       <c r="O1639" t="s">
         <v>426</v>
       </c>
@@ -79178,6 +80155,9 @@
       <c r="M1640" s="9">
         <v>5.31</v>
       </c>
+      <c r="N1640" s="9">
+        <v>0</v>
+      </c>
       <c r="O1640" t="s">
         <v>426</v>
       </c>
@@ -79225,6 +80205,9 @@
       <c r="M1641">
         <v>5.31</v>
       </c>
+      <c r="N1641">
+        <v>1</v>
+      </c>
       <c r="O1641" t="s">
         <v>426</v>
       </c>
@@ -79269,6 +80252,9 @@
       <c r="M1642">
         <v>5.31</v>
       </c>
+      <c r="N1642">
+        <v>1</v>
+      </c>
       <c r="O1642" t="s">
         <v>426</v>
       </c>
@@ -79313,6 +80299,9 @@
       <c r="M1643">
         <v>5.31</v>
       </c>
+      <c r="N1643">
+        <v>1</v>
+      </c>
       <c r="O1643" t="s">
         <v>426</v>
       </c>
@@ -79357,6 +80346,9 @@
       <c r="M1644">
         <v>5.31</v>
       </c>
+      <c r="N1644">
+        <v>1</v>
+      </c>
       <c r="O1644" t="s">
         <v>426</v>
       </c>
@@ -79401,6 +80393,9 @@
       <c r="M1645">
         <v>5.31</v>
       </c>
+      <c r="N1645">
+        <v>1</v>
+      </c>
       <c r="O1645" t="s">
         <v>426</v>
       </c>
@@ -79445,6 +80440,9 @@
       <c r="M1646">
         <v>5.31</v>
       </c>
+      <c r="N1646">
+        <v>1</v>
+      </c>
       <c r="O1646" t="s">
         <v>426</v>
       </c>
@@ -79489,6 +80487,9 @@
       <c r="M1647">
         <v>5.31</v>
       </c>
+      <c r="N1647">
+        <v>1</v>
+      </c>
       <c r="O1647" t="s">
         <v>426</v>
       </c>
@@ -79533,6 +80534,9 @@
       <c r="M1648">
         <v>5.31</v>
       </c>
+      <c r="N1648">
+        <v>1</v>
+      </c>
       <c r="O1648" t="s">
         <v>426</v>
       </c>
@@ -79577,6 +80581,9 @@
       <c r="M1649">
         <v>5.31</v>
       </c>
+      <c r="N1649">
+        <v>1</v>
+      </c>
       <c r="O1649" t="s">
         <v>426</v>
       </c>
@@ -79621,6 +80628,9 @@
       <c r="M1650">
         <v>5.31</v>
       </c>
+      <c r="N1650">
+        <v>1</v>
+      </c>
       <c r="O1650" t="s">
         <v>426</v>
       </c>
@@ -79665,6 +80675,9 @@
       <c r="M1651">
         <v>5.31</v>
       </c>
+      <c r="N1651">
+        <v>1</v>
+      </c>
       <c r="O1651" t="s">
         <v>426</v>
       </c>
@@ -79709,6 +80722,9 @@
       <c r="M1652">
         <v>5.31</v>
       </c>
+      <c r="N1652">
+        <v>1</v>
+      </c>
       <c r="O1652" t="s">
         <v>426</v>
       </c>
@@ -79857,6 +80873,9 @@
       <c r="M1657">
         <v>5.31</v>
       </c>
+      <c r="N1657">
+        <v>1</v>
+      </c>
       <c r="O1657" t="s">
         <v>427</v>
       </c>
@@ -79904,6 +80923,9 @@
       <c r="M1658">
         <v>5.31</v>
       </c>
+      <c r="N1658">
+        <v>1</v>
+      </c>
       <c r="O1658" t="s">
         <v>427</v>
       </c>
@@ -79951,6 +80973,9 @@
       <c r="M1659">
         <v>5.31</v>
       </c>
+      <c r="N1659">
+        <v>1</v>
+      </c>
       <c r="O1659" t="s">
         <v>427</v>
       </c>
@@ -79998,6 +81023,9 @@
       <c r="M1660">
         <v>5.31</v>
       </c>
+      <c r="N1660">
+        <v>1</v>
+      </c>
       <c r="O1660" t="s">
         <v>427</v>
       </c>
@@ -80045,6 +81073,9 @@
       <c r="M1661">
         <v>5.31</v>
       </c>
+      <c r="N1661">
+        <v>1</v>
+      </c>
       <c r="O1661" t="s">
         <v>427</v>
       </c>
@@ -80092,6 +81123,9 @@
       <c r="M1662">
         <v>5.31</v>
       </c>
+      <c r="N1662">
+        <v>1</v>
+      </c>
       <c r="O1662" t="s">
         <v>427</v>
       </c>
@@ -80139,6 +81173,9 @@
       <c r="M1663">
         <v>5.31</v>
       </c>
+      <c r="N1663">
+        <v>1</v>
+      </c>
       <c r="O1663" t="s">
         <v>427</v>
       </c>
@@ -80183,6 +81220,9 @@
       <c r="M1664">
         <v>5.31</v>
       </c>
+      <c r="N1664">
+        <v>1</v>
+      </c>
       <c r="O1664" t="s">
         <v>427</v>
       </c>
@@ -80227,6 +81267,9 @@
       <c r="M1665">
         <v>5.31</v>
       </c>
+      <c r="N1665">
+        <v>1</v>
+      </c>
       <c r="O1665" t="s">
         <v>427</v>
       </c>
@@ -80271,6 +81314,9 @@
       <c r="M1666">
         <v>5.31</v>
       </c>
+      <c r="N1666">
+        <v>1</v>
+      </c>
       <c r="O1666" t="s">
         <v>427</v>
       </c>
@@ -80315,6 +81361,9 @@
       <c r="M1667">
         <v>5.31</v>
       </c>
+      <c r="N1667">
+        <v>1</v>
+      </c>
       <c r="O1667" t="s">
         <v>427</v>
       </c>
@@ -80359,6 +81408,9 @@
       <c r="M1668">
         <v>5.31</v>
       </c>
+      <c r="N1668">
+        <v>1</v>
+      </c>
       <c r="O1668" t="s">
         <v>427</v>
       </c>
@@ -80403,6 +81455,9 @@
       <c r="M1669">
         <v>5.31</v>
       </c>
+      <c r="N1669">
+        <v>1</v>
+      </c>
       <c r="O1669" t="s">
         <v>427</v>
       </c>
@@ -80447,6 +81502,9 @@
       <c r="M1670">
         <v>5.31</v>
       </c>
+      <c r="N1670">
+        <v>1</v>
+      </c>
       <c r="O1670" t="s">
         <v>427</v>
       </c>
@@ -80491,6 +81549,9 @@
       <c r="M1671">
         <v>5.31</v>
       </c>
+      <c r="N1671">
+        <v>1</v>
+      </c>
       <c r="O1671" t="s">
         <v>427</v>
       </c>
@@ -80535,6 +81596,9 @@
       <c r="M1672">
         <v>5.31</v>
       </c>
+      <c r="N1672">
+        <v>1</v>
+      </c>
       <c r="O1672" t="s">
         <v>427</v>
       </c>
@@ -80579,6 +81643,9 @@
       <c r="M1673">
         <v>5.31</v>
       </c>
+      <c r="N1673">
+        <v>1</v>
+      </c>
       <c r="O1673" t="s">
         <v>427</v>
       </c>
@@ -80623,6 +81690,9 @@
       <c r="M1674">
         <v>5.31</v>
       </c>
+      <c r="N1674">
+        <v>1</v>
+      </c>
       <c r="O1674" t="s">
         <v>427</v>
       </c>
@@ -80667,6 +81737,9 @@
       <c r="M1675">
         <v>5.31</v>
       </c>
+      <c r="N1675">
+        <v>1</v>
+      </c>
       <c r="O1675" t="s">
         <v>427</v>
       </c>
@@ -80711,6 +81784,9 @@
       <c r="M1676">
         <v>5.31</v>
       </c>
+      <c r="N1676">
+        <v>1</v>
+      </c>
       <c r="O1676" t="s">
         <v>427</v>
       </c>
@@ -80755,6 +81831,9 @@
       <c r="M1677">
         <v>5.31</v>
       </c>
+      <c r="N1677">
+        <v>1</v>
+      </c>
       <c r="O1677" t="s">
         <v>427</v>
       </c>
@@ -80799,6 +81878,9 @@
       <c r="M1678">
         <v>5.31</v>
       </c>
+      <c r="N1678">
+        <v>1</v>
+      </c>
       <c r="O1678" t="s">
         <v>427</v>
       </c>
@@ -80846,6 +81928,9 @@
       <c r="M1679">
         <v>5.31</v>
       </c>
+      <c r="N1679">
+        <v>1</v>
+      </c>
       <c r="O1679" t="s">
         <v>427</v>
       </c>
@@ -80893,6 +81978,9 @@
       <c r="M1680">
         <v>5.31</v>
       </c>
+      <c r="N1680">
+        <v>1</v>
+      </c>
       <c r="O1680" t="s">
         <v>427</v>
       </c>
@@ -80940,6 +82028,9 @@
       <c r="M1681">
         <v>5.31</v>
       </c>
+      <c r="N1681">
+        <v>1</v>
+      </c>
       <c r="O1681" t="s">
         <v>427</v>
       </c>
@@ -80987,6 +82078,9 @@
       <c r="M1682">
         <v>5.31</v>
       </c>
+      <c r="N1682">
+        <v>1</v>
+      </c>
       <c r="O1682" t="s">
         <v>427</v>
       </c>
@@ -81034,6 +82128,9 @@
       <c r="M1683">
         <v>5.31</v>
       </c>
+      <c r="N1683">
+        <v>1</v>
+      </c>
       <c r="O1683" t="s">
         <v>427</v>
       </c>
@@ -81081,6 +82178,9 @@
       <c r="M1684">
         <v>5.31</v>
       </c>
+      <c r="N1684">
+        <v>1</v>
+      </c>
       <c r="O1684" t="s">
         <v>427</v>
       </c>
@@ -81125,6 +82225,9 @@
       <c r="M1685">
         <v>5.31</v>
       </c>
+      <c r="N1685">
+        <v>1</v>
+      </c>
       <c r="O1685" t="s">
         <v>427</v>
       </c>
@@ -81169,6 +82272,9 @@
       <c r="M1686">
         <v>5.31</v>
       </c>
+      <c r="N1686">
+        <v>1</v>
+      </c>
       <c r="O1686" t="s">
         <v>427</v>
       </c>
@@ -81213,6 +82319,9 @@
       <c r="M1687">
         <v>5.31</v>
       </c>
+      <c r="N1687">
+        <v>1</v>
+      </c>
       <c r="O1687" t="s">
         <v>427</v>
       </c>
@@ -81257,6 +82366,9 @@
       <c r="M1688">
         <v>5.31</v>
       </c>
+      <c r="N1688">
+        <v>1</v>
+      </c>
       <c r="O1688" t="s">
         <v>427</v>
       </c>
@@ -81301,6 +82413,9 @@
       <c r="M1689">
         <v>5.31</v>
       </c>
+      <c r="N1689">
+        <v>1</v>
+      </c>
       <c r="O1689" t="s">
         <v>427</v>
       </c>
@@ -81345,6 +82460,9 @@
       <c r="M1690">
         <v>5.31</v>
       </c>
+      <c r="N1690">
+        <v>1</v>
+      </c>
       <c r="O1690" t="s">
         <v>427</v>
       </c>
@@ -81389,6 +82507,9 @@
       <c r="M1691">
         <v>5.31</v>
       </c>
+      <c r="N1691">
+        <v>1</v>
+      </c>
       <c r="O1691" t="s">
         <v>427</v>
       </c>
@@ -81433,6 +82554,9 @@
       <c r="M1692">
         <v>5.31</v>
       </c>
+      <c r="N1692">
+        <v>1</v>
+      </c>
       <c r="O1692" t="s">
         <v>427</v>
       </c>
@@ -81477,6 +82601,9 @@
       <c r="M1693">
         <v>5.31</v>
       </c>
+      <c r="N1693">
+        <v>1</v>
+      </c>
       <c r="O1693" t="s">
         <v>427</v>
       </c>
@@ -81521,6 +82648,9 @@
       <c r="M1694">
         <v>5.31</v>
       </c>
+      <c r="N1694">
+        <v>1</v>
+      </c>
       <c r="O1694" t="s">
         <v>427</v>
       </c>
@@ -81565,6 +82695,9 @@
       <c r="M1695">
         <v>5.31</v>
       </c>
+      <c r="N1695">
+        <v>1</v>
+      </c>
       <c r="O1695" t="s">
         <v>427</v>
       </c>
@@ -81609,6 +82742,9 @@
       <c r="M1696">
         <v>5.31</v>
       </c>
+      <c r="N1696">
+        <v>1</v>
+      </c>
       <c r="O1696" t="s">
         <v>427</v>
       </c>
@@ -81653,6 +82789,9 @@
       <c r="M1697">
         <v>5.31</v>
       </c>
+      <c r="N1697">
+        <v>1</v>
+      </c>
       <c r="O1697" t="s">
         <v>427</v>
       </c>
@@ -81697,6 +82836,9 @@
       <c r="M1698">
         <v>5.31</v>
       </c>
+      <c r="N1698">
+        <v>1</v>
+      </c>
       <c r="O1698" t="s">
         <v>427</v>
       </c>
@@ -81845,6 +82987,9 @@
       <c r="M1703">
         <v>5.31</v>
       </c>
+      <c r="N1703">
+        <v>1</v>
+      </c>
       <c r="O1703" t="s">
         <v>428</v>
       </c>
@@ -81889,6 +83034,9 @@
       <c r="M1704">
         <v>5.31</v>
       </c>
+      <c r="N1704">
+        <v>1</v>
+      </c>
       <c r="O1704" t="s">
         <v>428</v>
       </c>
@@ -81933,6 +83081,9 @@
       <c r="M1705">
         <v>5.31</v>
       </c>
+      <c r="N1705">
+        <v>1</v>
+      </c>
       <c r="O1705" t="s">
         <v>428</v>
       </c>
@@ -81977,6 +83128,9 @@
       <c r="M1706">
         <v>5.31</v>
       </c>
+      <c r="N1706">
+        <v>1</v>
+      </c>
       <c r="O1706" t="s">
         <v>428</v>
       </c>
@@ -82021,6 +83175,9 @@
       <c r="M1707">
         <v>5.31</v>
       </c>
+      <c r="N1707">
+        <v>1</v>
+      </c>
       <c r="O1707" t="s">
         <v>428</v>
       </c>
@@ -82065,6 +83222,9 @@
       <c r="M1708">
         <v>5.31</v>
       </c>
+      <c r="N1708">
+        <v>1</v>
+      </c>
       <c r="O1708" t="s">
         <v>428</v>
       </c>
@@ -82109,6 +83269,9 @@
       <c r="M1709">
         <v>5.31</v>
       </c>
+      <c r="N1709">
+        <v>1</v>
+      </c>
       <c r="O1709" t="s">
         <v>428</v>
       </c>
@@ -82156,6 +83319,9 @@
       <c r="M1710">
         <v>5.31</v>
       </c>
+      <c r="N1710">
+        <v>1</v>
+      </c>
       <c r="O1710" t="s">
         <v>428</v>
       </c>
@@ -82203,6 +83369,9 @@
       <c r="M1711">
         <v>5.31</v>
       </c>
+      <c r="N1711">
+        <v>1</v>
+      </c>
       <c r="O1711" t="s">
         <v>428</v>
       </c>
@@ -82250,6 +83419,9 @@
       <c r="M1712">
         <v>5.31</v>
       </c>
+      <c r="N1712">
+        <v>1</v>
+      </c>
       <c r="O1712" t="s">
         <v>428</v>
       </c>
@@ -82297,6 +83469,9 @@
       <c r="M1713">
         <v>5.31</v>
       </c>
+      <c r="N1713">
+        <v>1</v>
+      </c>
       <c r="O1713" t="s">
         <v>428</v>
       </c>
@@ -82344,6 +83519,9 @@
       <c r="M1714">
         <v>5.31</v>
       </c>
+      <c r="N1714">
+        <v>1</v>
+      </c>
       <c r="O1714" t="s">
         <v>428</v>
       </c>
@@ -82441,6 +83619,9 @@
       <c r="M1716">
         <v>5.31</v>
       </c>
+      <c r="N1716">
+        <v>1</v>
+      </c>
       <c r="O1716" t="s">
         <v>428</v>
       </c>
@@ -82485,6 +83666,9 @@
       <c r="M1717">
         <v>5.31</v>
       </c>
+      <c r="N1717">
+        <v>1</v>
+      </c>
       <c r="O1717" t="s">
         <v>428</v>
       </c>
@@ -82529,6 +83713,9 @@
       <c r="M1718">
         <v>5.31</v>
       </c>
+      <c r="N1718">
+        <v>1</v>
+      </c>
       <c r="O1718" t="s">
         <v>428</v>
       </c>
@@ -82573,6 +83760,9 @@
       <c r="M1719" s="9">
         <v>5.31</v>
       </c>
+      <c r="N1719" s="9">
+        <v>0</v>
+      </c>
       <c r="O1719" t="s">
         <v>428</v>
       </c>
@@ -82620,6 +83810,9 @@
       <c r="M1720">
         <v>5.31</v>
       </c>
+      <c r="N1720">
+        <v>1</v>
+      </c>
       <c r="O1720" t="s">
         <v>428</v>
       </c>
@@ -82664,6 +83857,9 @@
       <c r="M1721">
         <v>5.31</v>
       </c>
+      <c r="N1721">
+        <v>1</v>
+      </c>
       <c r="O1721" t="s">
         <v>428</v>
       </c>
@@ -82708,6 +83904,9 @@
       <c r="M1722">
         <v>5.31</v>
       </c>
+      <c r="N1722">
+        <v>1</v>
+      </c>
       <c r="O1722" t="s">
         <v>428</v>
       </c>
@@ -82752,6 +83951,9 @@
       <c r="M1723">
         <v>5.31</v>
       </c>
+      <c r="N1723">
+        <v>1</v>
+      </c>
       <c r="O1723" t="s">
         <v>428</v>
       </c>
@@ -82796,6 +83998,9 @@
       <c r="M1724">
         <v>5.31</v>
       </c>
+      <c r="N1724">
+        <v>1</v>
+      </c>
       <c r="O1724" t="s">
         <v>428</v>
       </c>
@@ -82843,6 +84048,9 @@
       <c r="M1725">
         <v>5.31</v>
       </c>
+      <c r="N1725">
+        <v>1</v>
+      </c>
       <c r="O1725" t="s">
         <v>428</v>
       </c>
@@ -82890,6 +84098,9 @@
       <c r="M1726">
         <v>5.31</v>
       </c>
+      <c r="N1726">
+        <v>1</v>
+      </c>
       <c r="O1726" t="s">
         <v>428</v>
       </c>
@@ -82937,6 +84148,9 @@
       <c r="M1727">
         <v>5.31</v>
       </c>
+      <c r="N1727">
+        <v>1</v>
+      </c>
       <c r="O1727" t="s">
         <v>428</v>
       </c>
@@ -82981,6 +84195,9 @@
       <c r="M1728">
         <v>5.31</v>
       </c>
+      <c r="N1728">
+        <v>1</v>
+      </c>
       <c r="O1728" t="s">
         <v>428</v>
       </c>
@@ -83025,6 +84242,9 @@
       <c r="M1729">
         <v>5.31</v>
       </c>
+      <c r="N1729">
+        <v>1</v>
+      </c>
       <c r="O1729" t="s">
         <v>428</v>
       </c>
@@ -83069,6 +84289,9 @@
       <c r="M1730">
         <v>5.31</v>
       </c>
+      <c r="N1730">
+        <v>1</v>
+      </c>
       <c r="O1730" t="s">
         <v>428</v>
       </c>
@@ -83113,6 +84336,9 @@
       <c r="M1731">
         <v>5.31</v>
       </c>
+      <c r="N1731">
+        <v>1</v>
+      </c>
       <c r="O1731" t="s">
         <v>428</v>
       </c>
@@ -83157,6 +84383,9 @@
       <c r="M1732">
         <v>5.31</v>
       </c>
+      <c r="N1732">
+        <v>1</v>
+      </c>
       <c r="O1732" t="s">
         <v>428</v>
       </c>
@@ -83201,6 +84430,9 @@
       <c r="M1733">
         <v>5.31</v>
       </c>
+      <c r="N1733">
+        <v>1</v>
+      </c>
       <c r="O1733" t="s">
         <v>428</v>
       </c>
@@ -83245,6 +84477,9 @@
       <c r="M1734">
         <v>5.31</v>
       </c>
+      <c r="N1734">
+        <v>1</v>
+      </c>
       <c r="O1734" t="s">
         <v>428</v>
       </c>
@@ -83289,6 +84524,9 @@
       <c r="M1735">
         <v>5.31</v>
       </c>
+      <c r="N1735">
+        <v>1</v>
+      </c>
       <c r="O1735" t="s">
         <v>428</v>
       </c>
@@ -83383,6 +84621,9 @@
       <c r="M1737">
         <v>5.31</v>
       </c>
+      <c r="N1737">
+        <v>1</v>
+      </c>
       <c r="O1737" t="s">
         <v>428</v>
       </c>
@@ -83477,6 +84718,9 @@
       <c r="M1739">
         <v>5.31</v>
       </c>
+      <c r="N1739">
+        <v>1</v>
+      </c>
       <c r="O1739" t="s">
         <v>428</v>
       </c>
@@ -83521,6 +84765,9 @@
       <c r="M1740">
         <v>5.31</v>
       </c>
+      <c r="N1740">
+        <v>1</v>
+      </c>
       <c r="O1740" t="s">
         <v>428</v>
       </c>
@@ -83615,6 +84862,9 @@
       <c r="M1742">
         <v>5.31</v>
       </c>
+      <c r="N1742">
+        <v>1</v>
+      </c>
       <c r="O1742" t="s">
         <v>428</v>
       </c>
@@ -83659,6 +84909,9 @@
       <c r="M1743">
         <v>5.31</v>
       </c>
+      <c r="N1743">
+        <v>1</v>
+      </c>
       <c r="O1743" t="s">
         <v>428</v>
       </c>
@@ -83703,6 +84956,9 @@
       <c r="M1744">
         <v>5.31</v>
       </c>
+      <c r="N1744">
+        <v>1</v>
+      </c>
       <c r="O1744" t="s">
         <v>428</v>
       </c>
@@ -83851,6 +85107,9 @@
       <c r="M1749">
         <v>5.31</v>
       </c>
+      <c r="N1749">
+        <v>1</v>
+      </c>
       <c r="O1749" t="s">
         <v>429</v>
       </c>
@@ -83898,6 +85157,9 @@
       <c r="M1750">
         <v>5.31</v>
       </c>
+      <c r="N1750">
+        <v>1</v>
+      </c>
       <c r="O1750" t="s">
         <v>429</v>
       </c>
@@ -83945,6 +85207,9 @@
       <c r="M1751">
         <v>5.31</v>
       </c>
+      <c r="N1751">
+        <v>1</v>
+      </c>
       <c r="O1751" t="s">
         <v>429</v>
       </c>
@@ -83992,6 +85257,9 @@
       <c r="M1752">
         <v>5.31</v>
       </c>
+      <c r="N1752">
+        <v>1</v>
+      </c>
       <c r="O1752" t="s">
         <v>429</v>
       </c>
@@ -84039,6 +85307,9 @@
       <c r="M1753">
         <v>5.31</v>
       </c>
+      <c r="N1753">
+        <v>1</v>
+      </c>
       <c r="O1753" t="s">
         <v>429</v>
       </c>
@@ -84086,6 +85357,9 @@
       <c r="M1754">
         <v>5.31</v>
       </c>
+      <c r="N1754">
+        <v>1</v>
+      </c>
       <c r="O1754" t="s">
         <v>429</v>
       </c>
@@ -84133,6 +85407,9 @@
       <c r="M1755">
         <v>5.31</v>
       </c>
+      <c r="N1755">
+        <v>1</v>
+      </c>
       <c r="O1755" t="s">
         <v>429</v>
       </c>
@@ -84180,6 +85457,9 @@
       <c r="M1756">
         <v>5.31</v>
       </c>
+      <c r="N1756">
+        <v>1</v>
+      </c>
       <c r="O1756" t="s">
         <v>429</v>
       </c>
@@ -84227,6 +85507,9 @@
       <c r="M1757">
         <v>5.31</v>
       </c>
+      <c r="N1757">
+        <v>1</v>
+      </c>
       <c r="O1757" t="s">
         <v>429</v>
       </c>
@@ -84274,6 +85557,9 @@
       <c r="M1758">
         <v>5.31</v>
       </c>
+      <c r="N1758">
+        <v>1</v>
+      </c>
       <c r="O1758" t="s">
         <v>429</v>
       </c>
@@ -84321,6 +85607,9 @@
       <c r="M1759">
         <v>5.31</v>
       </c>
+      <c r="N1759">
+        <v>1</v>
+      </c>
       <c r="O1759" t="s">
         <v>429</v>
       </c>
@@ -84368,6 +85657,9 @@
       <c r="M1760">
         <v>5.31</v>
       </c>
+      <c r="N1760">
+        <v>1</v>
+      </c>
       <c r="O1760" t="s">
         <v>429</v>
       </c>
@@ -84415,6 +85707,9 @@
       <c r="M1761">
         <v>5.31</v>
       </c>
+      <c r="N1761">
+        <v>1</v>
+      </c>
       <c r="O1761" t="s">
         <v>429</v>
       </c>
@@ -84462,6 +85757,9 @@
       <c r="M1762">
         <v>5.31</v>
       </c>
+      <c r="N1762">
+        <v>1</v>
+      </c>
       <c r="O1762" t="s">
         <v>429</v>
       </c>
@@ -84509,6 +85807,9 @@
       <c r="M1763">
         <v>5.31</v>
       </c>
+      <c r="N1763">
+        <v>1</v>
+      </c>
       <c r="O1763" t="s">
         <v>429</v>
       </c>
@@ -84556,6 +85857,9 @@
       <c r="M1764">
         <v>5.31</v>
       </c>
+      <c r="N1764">
+        <v>1</v>
+      </c>
       <c r="O1764" t="s">
         <v>429</v>
       </c>
@@ -84603,6 +85907,9 @@
       <c r="M1765">
         <v>5.31</v>
       </c>
+      <c r="N1765">
+        <v>1</v>
+      </c>
       <c r="O1765" t="s">
         <v>429</v>
       </c>
@@ -84650,6 +85957,9 @@
       <c r="M1766">
         <v>5.31</v>
       </c>
+      <c r="N1766">
+        <v>1</v>
+      </c>
       <c r="O1766" t="s">
         <v>429</v>
       </c>
@@ -84697,6 +86007,9 @@
       <c r="M1767">
         <v>5.31</v>
       </c>
+      <c r="N1767">
+        <v>1</v>
+      </c>
       <c r="O1767" t="s">
         <v>429</v>
       </c>
@@ -84744,6 +86057,9 @@
       <c r="M1768">
         <v>5.31</v>
       </c>
+      <c r="N1768">
+        <v>1</v>
+      </c>
       <c r="O1768" t="s">
         <v>429</v>
       </c>
@@ -84791,6 +86107,9 @@
       <c r="M1769">
         <v>5.31</v>
       </c>
+      <c r="N1769">
+        <v>1</v>
+      </c>
       <c r="O1769" t="s">
         <v>429</v>
       </c>
@@ -84838,6 +86157,9 @@
       <c r="M1770">
         <v>5.31</v>
       </c>
+      <c r="N1770">
+        <v>1</v>
+      </c>
       <c r="O1770" t="s">
         <v>429</v>
       </c>
@@ -84885,6 +86207,9 @@
       <c r="M1771">
         <v>5.31</v>
       </c>
+      <c r="N1771">
+        <v>1</v>
+      </c>
       <c r="O1771" t="s">
         <v>429</v>
       </c>
@@ -84932,6 +86257,9 @@
       <c r="M1772">
         <v>5.31</v>
       </c>
+      <c r="N1772">
+        <v>1</v>
+      </c>
       <c r="O1772" t="s">
         <v>429</v>
       </c>
@@ -84979,6 +86307,9 @@
       <c r="M1773">
         <v>5.31</v>
       </c>
+      <c r="N1773">
+        <v>1</v>
+      </c>
       <c r="O1773" t="s">
         <v>429</v>
       </c>
@@ -85026,6 +86357,9 @@
       <c r="M1774">
         <v>5.31</v>
       </c>
+      <c r="N1774">
+        <v>1</v>
+      </c>
       <c r="O1774" t="s">
         <v>429</v>
       </c>
@@ -85073,6 +86407,9 @@
       <c r="M1775">
         <v>5.31</v>
       </c>
+      <c r="N1775">
+        <v>1</v>
+      </c>
       <c r="O1775" t="s">
         <v>429</v>
       </c>
@@ -85120,6 +86457,9 @@
       <c r="M1776">
         <v>5.31</v>
       </c>
+      <c r="N1776">
+        <v>1</v>
+      </c>
       <c r="O1776" t="s">
         <v>429</v>
       </c>
@@ -85167,6 +86507,9 @@
       <c r="M1777">
         <v>5.31</v>
       </c>
+      <c r="N1777">
+        <v>1</v>
+      </c>
       <c r="O1777" t="s">
         <v>429</v>
       </c>
@@ -85214,6 +86557,9 @@
       <c r="M1778">
         <v>5.31</v>
       </c>
+      <c r="N1778">
+        <v>1</v>
+      </c>
       <c r="O1778" t="s">
         <v>429</v>
       </c>
@@ -85261,6 +86607,9 @@
       <c r="M1779">
         <v>5.31</v>
       </c>
+      <c r="N1779">
+        <v>1</v>
+      </c>
       <c r="O1779" t="s">
         <v>429</v>
       </c>
@@ -85308,6 +86657,9 @@
       <c r="M1780">
         <v>5.31</v>
       </c>
+      <c r="N1780">
+        <v>1</v>
+      </c>
       <c r="O1780" t="s">
         <v>429</v>
       </c>
@@ -85355,6 +86707,9 @@
       <c r="M1781">
         <v>5.31</v>
       </c>
+      <c r="N1781">
+        <v>1</v>
+      </c>
       <c r="O1781" t="s">
         <v>429</v>
       </c>
@@ -85402,6 +86757,9 @@
       <c r="M1782">
         <v>5.31</v>
       </c>
+      <c r="N1782">
+        <v>1</v>
+      </c>
       <c r="O1782" t="s">
         <v>429</v>
       </c>
@@ -85449,6 +86807,9 @@
       <c r="M1783">
         <v>5.31</v>
       </c>
+      <c r="N1783">
+        <v>1</v>
+      </c>
       <c r="O1783" t="s">
         <v>429</v>
       </c>
@@ -85496,6 +86857,9 @@
       <c r="M1784">
         <v>5.31</v>
       </c>
+      <c r="N1784">
+        <v>1</v>
+      </c>
       <c r="O1784" t="s">
         <v>429</v>
       </c>
@@ -85543,6 +86907,9 @@
       <c r="M1785">
         <v>5.31</v>
       </c>
+      <c r="N1785">
+        <v>1</v>
+      </c>
       <c r="O1785" t="s">
         <v>429</v>
       </c>
@@ -85590,6 +86957,9 @@
       <c r="M1786">
         <v>5.31</v>
       </c>
+      <c r="N1786">
+        <v>1</v>
+      </c>
       <c r="O1786" t="s">
         <v>429</v>
       </c>
@@ -85637,6 +87007,9 @@
       <c r="M1787">
         <v>5.31</v>
       </c>
+      <c r="N1787">
+        <v>1</v>
+      </c>
       <c r="O1787" t="s">
         <v>429</v>
       </c>
@@ -85684,6 +87057,9 @@
       <c r="M1788">
         <v>5.31</v>
       </c>
+      <c r="N1788">
+        <v>1</v>
+      </c>
       <c r="O1788" t="s">
         <v>429</v>
       </c>
@@ -85731,6 +87107,9 @@
       <c r="M1789">
         <v>5.31</v>
       </c>
+      <c r="N1789">
+        <v>1</v>
+      </c>
       <c r="O1789" t="s">
         <v>429</v>
       </c>
@@ -85778,6 +87157,9 @@
       <c r="M1790">
         <v>5.31</v>
       </c>
+      <c r="N1790">
+        <v>1</v>
+      </c>
       <c r="O1790" t="s">
         <v>429</v>
       </c>
@@ -86470,6 +87852,9 @@
       <c r="M1814" s="9">
         <v>5.31</v>
       </c>
+      <c r="N1814" s="9">
+        <v>0</v>
+      </c>
       <c r="O1814" t="s">
         <v>430</v>
       </c>
@@ -86503,6 +87888,9 @@
       </c>
       <c r="M1815" s="9">
         <v>5.31</v>
+      </c>
+      <c r="N1815" s="9">
+        <v>0</v>
       </c>
       <c r="O1815" t="s">
         <v>430</v>

</xml_diff>

<commit_message>
Finishing the Site C check in with Mattl
Adding more detail for the site c and cleaning up Site B and Site C comparison notes and usgs database references
</commit_message>
<xml_diff>
--- a/data/thesis_sediment master (raw).xlsx
+++ b/data/thesis_sediment master (raw).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mailsfsu-my.sharepoint.com/personal/924318106_sfsu_edu/Documents/ProjectData/GitHub/DepositionSFB/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1445" documentId="8_{625E32F6-7E88-4DA8-AE14-1AD01B36A6CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BBF7FC61-E671-4955-B961-F6948BE73005}"/>
+  <xr:revisionPtr revIDLastSave="1446" documentId="8_{625E32F6-7E88-4DA8-AE14-1AD01B36A6CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E33B2F5E-71B8-41F6-B697-3215BC61A37E}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13152" xr2:uid="{7E299392-FF5E-4B95-B4B7-FEDF7BC05BEF}"/>
+    <workbookView xWindow="-14505" yWindow="-3960" windowWidth="14610" windowHeight="16305" xr2:uid="{7E299392-FF5E-4B95-B4B7-FEDF7BC05BEF}"/>
   </bookViews>
   <sheets>
     <sheet name="sediment master (raw)" sheetId="1" r:id="rId1"/>
@@ -90262,9 +90262,6 @@
       <c r="M1897">
         <v>5.31</v>
       </c>
-      <c r="N1897">
-        <v>0.75</v>
-      </c>
       <c r="O1897" t="s">
         <v>432</v>
       </c>
@@ -90948,9 +90945,6 @@
       <c r="M1920">
         <v>5.31</v>
       </c>
-      <c r="N1920">
-        <v>0.75</v>
-      </c>
       <c r="O1920" t="s">
         <v>432</v>
       </c>
@@ -91074,9 +91068,6 @@
       </c>
       <c r="M1924" s="9">
         <v>5.31</v>
-      </c>
-      <c r="N1924" s="9">
-        <v>0.5</v>
       </c>
       <c r="O1924" t="s">
         <v>432</v>

</xml_diff>